<commit_message>
update perhitungan biaya bunga
</commit_message>
<xml_diff>
--- a/data/file/tabel_mortalita.xlsx
+++ b/data/file/tabel_mortalita.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Kerjaan Arya\KKA VAB\Aplikasi\imbalan-pasca-kerja-app\data\file\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aryax punya\2026\KKA VAB\Aplikasi\imbalan-pasca-kerja-app\data\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42389C61-2A14-42AE-AD69-7E1F10D9CA46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F441F44-53BE-44DE-826C-2BFCCA24AACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2C21EB3D-DA47-424B-AC62-B057914736D2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2C21EB3D-DA47-424B-AC62-B057914736D2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -583,45 +583,46 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C72DD34E-A333-46DB-95FC-B843EE1C81C8}">
   <dimension ref="A1:AX120"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="20.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="6" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="33" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="38" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="39" max="41" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="33" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="38" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="39" max="41" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="10" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="44" max="45" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="15.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="C1">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -663,12 +664,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="3">
-        <v>0.93784486447342408</v>
+        <v>0.93904586232916898</v>
       </c>
       <c r="H2">
         <v>2</v>
@@ -707,12 +708,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="3">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
@@ -751,7 +752,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -792,12 +793,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:50" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>30</v>
       </c>
@@ -941,7 +942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>1</v>
       </c>
@@ -1084,7 +1085,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>13</v>
       </c>
@@ -1114,40 +1115,40 @@
         <v>0</v>
       </c>
       <c r="K8" s="12">
-        <v>7229969.5934085008</v>
+        <v>8325097.5736416606</v>
       </c>
       <c r="L8" s="12">
         <v>0</v>
       </c>
       <c r="M8" s="12">
-        <v>1400.3280791679515</v>
+        <v>1613.4687496331269</v>
       </c>
       <c r="N8" s="12">
-        <v>70.009752366763564</v>
+        <v>80.665773466775519</v>
       </c>
       <c r="O8" s="12">
         <v>0</v>
       </c>
       <c r="P8" s="12">
-        <v>142931.87615939724</v>
+        <v>465344.81742319983</v>
       </c>
       <c r="Q8" s="12">
-        <v>7134.8782793052369</v>
+        <v>23212.119656511517</v>
       </c>
       <c r="R8" s="12">
-        <v>2999192.8754028431</v>
+        <v>1356161.511816124</v>
       </c>
       <c r="S8" s="12">
-        <v>4016835.5136271138</v>
+        <v>15990839.339348922</v>
       </c>
       <c r="T8" s="12">
-        <v>200394.54641248754</v>
+        <v>797280.53516904812</v>
       </c>
       <c r="U8" s="12">
-        <v>48167640.489707701</v>
+        <v>26559258.620586243</v>
       </c>
       <c r="V8" s="13">
-        <v>0</v>
+        <v>0.68173499308842878</v>
       </c>
       <c r="W8" s="13"/>
       <c r="AA8" s="1" t="s">
@@ -1160,7 +1161,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>14</v>
       </c>
@@ -1190,40 +1191,40 @@
         <v>0</v>
       </c>
       <c r="K9" s="12">
-        <v>7050332.5808958877</v>
+        <v>8206807.0764537863</v>
       </c>
       <c r="L9" s="12">
         <v>0</v>
       </c>
       <c r="M9" s="12">
-        <v>1570.3644144801367</v>
+        <v>1829.123227620787</v>
       </c>
       <c r="N9" s="12">
-        <v>78.509642559068709</v>
+        <v>91.446169737957021</v>
       </c>
       <c r="O9" s="12">
         <v>0</v>
       </c>
       <c r="P9" s="12">
-        <v>141531.54808022929</v>
+        <v>463731.34867356677</v>
       </c>
       <c r="Q9" s="12">
-        <v>7064.8685269384723</v>
+        <v>23131.453883044742</v>
       </c>
       <c r="R9" s="12">
-        <v>2999192.8754028431</v>
+        <v>1356161.511816124</v>
       </c>
       <c r="S9" s="12">
-        <v>3873903.6374677168</v>
+        <v>15525494.521925721</v>
       </c>
       <c r="T9" s="12">
-        <v>193259.66813318231</v>
+        <v>774068.41551253654</v>
       </c>
       <c r="U9" s="12">
-        <v>45168447.614304855</v>
+        <v>25203097.108770121</v>
       </c>
       <c r="V9" s="13">
-        <v>0</v>
+        <v>0.68187818614376261</v>
       </c>
       <c r="W9" s="13"/>
       <c r="X9" s="5">
@@ -1305,7 +1306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>15</v>
       </c>
@@ -1335,40 +1336,40 @@
         <v>0</v>
       </c>
       <c r="K10" s="12">
-        <v>6874942.2505563274</v>
+        <v>8089942.4678461915</v>
       </c>
       <c r="L10" s="12">
         <v>0</v>
       </c>
       <c r="M10" s="12">
-        <v>1797.609644207412</v>
+        <v>2116.6530049813482</v>
       </c>
       <c r="N10" s="12">
-        <v>89.868954960718099</v>
+        <v>105.81907712005425</v>
       </c>
       <c r="O10" s="12">
         <v>0</v>
       </c>
       <c r="P10" s="12">
-        <v>139961.18366574915</v>
+        <v>461902.22544594592</v>
       </c>
       <c r="Q10" s="12">
-        <v>6986.3588843794032</v>
+        <v>23040.007713306783</v>
       </c>
       <c r="R10" s="12">
-        <v>2999192.8754028431</v>
+        <v>1356161.511816124</v>
       </c>
       <c r="S10" s="12">
-        <v>3732372.0893874867</v>
+        <v>15061763.173252154</v>
       </c>
       <c r="T10" s="12">
-        <v>186194.79960624382</v>
+        <v>750936.96162949188</v>
       </c>
       <c r="U10" s="12">
-        <v>42169254.738902025</v>
+        <v>23846935.596953992</v>
       </c>
       <c r="V10" s="13">
-        <v>0</v>
+        <v>0.68204289769955351</v>
       </c>
       <c r="W10" s="13"/>
       <c r="X10" s="5">
@@ -1450,7 +1451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>16</v>
       </c>
@@ -1480,40 +1481,40 @@
         <v>0</v>
       </c>
       <c r="K11" s="12">
-        <v>6703633.4599888446</v>
+        <v>7974406.9945550496</v>
       </c>
       <c r="L11" s="12">
         <v>0</v>
       </c>
       <c r="M11" s="12">
-        <v>2012.4916649428094</v>
+        <v>2395.5217975560008</v>
       </c>
       <c r="N11" s="12">
-        <v>100.60976616242493</v>
+        <v>119.7584527118775</v>
       </c>
       <c r="O11" s="12">
         <v>0</v>
       </c>
       <c r="P11" s="12">
-        <v>138163.57402154175</v>
+        <v>459785.57244096458</v>
       </c>
       <c r="Q11" s="12">
-        <v>6896.4899294186853</v>
+        <v>22934.188636186729</v>
       </c>
       <c r="R11" s="12">
-        <v>2999192.8754028431</v>
+        <v>1356161.511816124</v>
       </c>
       <c r="S11" s="12">
-        <v>3592410.905721738</v>
+        <v>14599860.947806207</v>
       </c>
       <c r="T11" s="12">
-        <v>179208.44072186443</v>
+        <v>727896.95391618507</v>
       </c>
       <c r="U11" s="12">
-        <v>39170061.863499172</v>
+        <v>22490774.08513787</v>
       </c>
       <c r="V11" s="13">
-        <v>0</v>
+        <v>0.68223630920646228</v>
       </c>
       <c r="W11" s="13"/>
       <c r="X11" s="5">
@@ -1595,7 +1596,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>17</v>
       </c>
@@ -1625,40 +1626,40 @@
         <v>0</v>
       </c>
       <c r="K12" s="12">
-        <v>6536318.7092507742</v>
+        <v>7860191.2998683061</v>
       </c>
       <c r="L12" s="12">
         <v>0</v>
       </c>
       <c r="M12" s="12">
-        <v>2342.0514385226743</v>
+        <v>2818.2156642679538</v>
       </c>
       <c r="N12" s="12">
-        <v>117.08199095874346</v>
+        <v>140.88601791416858</v>
       </c>
       <c r="O12" s="12">
         <v>0</v>
       </c>
       <c r="P12" s="12">
-        <v>136151.0823565989</v>
+        <v>457390.05064340861</v>
       </c>
       <c r="Q12" s="12">
-        <v>6795.8801632562599</v>
+        <v>22814.430183474851</v>
       </c>
       <c r="R12" s="12">
-        <v>2999192.8754028431</v>
+        <v>1356161.511816124</v>
       </c>
       <c r="S12" s="12">
-        <v>3454247.3317001956</v>
+        <v>14140075.375365244</v>
       </c>
       <c r="T12" s="12">
-        <v>172311.95079244577</v>
+        <v>704962.7652799983</v>
       </c>
       <c r="U12" s="12">
-        <v>36170868.988096334</v>
+        <v>21134612.573321749</v>
       </c>
       <c r="V12" s="13">
-        <v>0</v>
+        <v>0.68245844615147166</v>
       </c>
       <c r="W12" s="13"/>
       <c r="X12" s="5">
@@ -1740,7 +1741,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>18</v>
       </c>
@@ -1770,40 +1771,40 @@
         <v>0</v>
       </c>
       <c r="K13" s="12">
-        <v>6372778.3084448492</v>
+        <v>7747123.2490627524</v>
       </c>
       <c r="L13" s="12">
         <v>0</v>
       </c>
       <c r="M13" s="12">
-        <v>2653.7383463731876</v>
+        <v>3228.105009770622</v>
       </c>
       <c r="N13" s="12">
-        <v>132.65981572445477</v>
+        <v>161.37228311171938</v>
       </c>
       <c r="O13" s="12">
         <v>0</v>
       </c>
       <c r="P13" s="12">
-        <v>133809.03091807623</v>
+        <v>454571.83497914061</v>
       </c>
       <c r="Q13" s="12">
-        <v>6678.7981722975173</v>
+        <v>22673.544165560685</v>
       </c>
       <c r="R13" s="12">
-        <v>2999192.8754028431</v>
+        <v>1356161.511816124</v>
       </c>
       <c r="S13" s="12">
-        <v>3318096.2493435973</v>
+        <v>13682685.324721836</v>
       </c>
       <c r="T13" s="12">
-        <v>165516.07062918952</v>
+        <v>682148.33509652351</v>
       </c>
       <c r="U13" s="12">
-        <v>33171676.1126935</v>
+        <v>19778451.061505627</v>
       </c>
       <c r="V13" s="13">
-        <v>0</v>
+        <v>0.68272367962776348</v>
       </c>
       <c r="W13" s="13"/>
       <c r="X13" s="5">
@@ -1885,7 +1886,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>19</v>
       </c>
@@ -1915,40 +1916,40 @@
         <v>0</v>
       </c>
       <c r="K14" s="12">
-        <v>6212938.154183127</v>
+        <v>7635200.4540761588</v>
       </c>
       <c r="L14" s="12">
         <v>0</v>
       </c>
       <c r="M14" s="12">
-        <v>2827.8429590725232</v>
+        <v>3477.4156165045511</v>
       </c>
       <c r="N14" s="12">
-        <v>141.36058178569297</v>
+        <v>173.83196371730722</v>
       </c>
       <c r="O14" s="12">
         <v>0</v>
       </c>
       <c r="P14" s="12">
-        <v>131155.29257170303</v>
+        <v>451343.72996937</v>
       </c>
       <c r="Q14" s="12">
-        <v>6546.1383565730621</v>
+        <v>22512.171882448965</v>
       </c>
       <c r="R14" s="12">
-        <v>2999192.8754028431</v>
+        <v>1356161.511816124</v>
       </c>
       <c r="S14" s="12">
-        <v>3184287.2184255207</v>
+        <v>13228113.489742696</v>
       </c>
       <c r="T14" s="12">
-        <v>158837.27245689195</v>
+        <v>659474.79093096289</v>
       </c>
       <c r="U14" s="12">
-        <v>30172483.237290654</v>
+        <v>18422289.549689498</v>
       </c>
       <c r="V14" s="13">
-        <v>0</v>
+        <v>0.68303206228925573</v>
       </c>
       <c r="W14" s="13"/>
       <c r="X14" s="5">
@@ -2030,7 +2031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>20</v>
       </c>
@@ -2041,7 +2042,7 @@
         <v>2.4499999999999999E-5</v>
       </c>
       <c r="D15" s="11">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E15" s="10">
         <v>0</v>
@@ -2050,52 +2051,52 @@
         <v>9976084.6089028642</v>
       </c>
       <c r="G15" s="12">
-        <v>4766.0160374916704</v>
+        <v>4863.7804690299699</v>
       </c>
       <c r="H15" s="12">
-        <v>238.245336683499</v>
+        <v>243.13242051290399</v>
       </c>
       <c r="I15" s="12">
-        <v>498675.91455389699</v>
+        <v>99735.182910779506</v>
       </c>
       <c r="J15" s="12">
         <v>0</v>
       </c>
       <c r="K15" s="12">
-        <v>6056852.5612365287</v>
+        <v>7524578.4344527898</v>
       </c>
       <c r="L15" s="12">
         <v>0</v>
       </c>
       <c r="M15" s="12">
-        <v>2802.2564656292384</v>
+        <v>3554.9984513962445</v>
       </c>
       <c r="N15" s="12">
-        <v>140.08021162235056</v>
+        <v>177.70855076852942</v>
       </c>
       <c r="O15" s="12">
-        <v>293204.59579227207</v>
+        <v>72897.702323364792</v>
       </c>
       <c r="P15" s="12">
-        <v>128327.4496126305</v>
+        <v>447866.31435286539</v>
       </c>
       <c r="Q15" s="12">
-        <v>6404.7777747873688</v>
+        <v>22338.339918731657</v>
       </c>
       <c r="R15" s="12">
-        <v>2999192.8754028431</v>
+        <v>1356161.511816124</v>
       </c>
       <c r="S15" s="12">
-        <v>3053131.9258538177</v>
+        <v>12776769.759773327</v>
       </c>
       <c r="T15" s="12">
-        <v>152291.13410031892</v>
+        <v>636962.61904851382</v>
       </c>
       <c r="U15" s="12">
-        <v>27173290.361887809</v>
+        <v>17066128.037873376</v>
       </c>
       <c r="V15" s="13">
-        <v>0</v>
+        <v>0.68336929748975306</v>
       </c>
       <c r="W15" s="13"/>
       <c r="X15" s="5">
@@ -2177,7 +2178,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>21</v>
       </c>
@@ -2188,61 +2189,61 @@
         <v>2.4499999999999999E-5</v>
       </c>
       <c r="D16" s="11">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E16" s="10">
         <v>0</v>
       </c>
       <c r="F16" s="12">
-        <v>9472404.4329747912</v>
+        <v>9871242.5131025407</v>
       </c>
       <c r="G16" s="12">
-        <v>4525.38578119879</v>
+        <v>4812.6653313906199</v>
       </c>
       <c r="H16" s="12">
-        <v>226.21662423776701</v>
+        <v>240.577258490638</v>
       </c>
       <c r="I16" s="12">
-        <v>473498.38426817302</v>
+        <v>98687.031655921106</v>
       </c>
       <c r="J16" s="12">
         <v>0</v>
       </c>
       <c r="K16" s="12">
-        <v>5609335.9919107147</v>
+        <v>7341249.3236715542</v>
       </c>
       <c r="L16" s="12">
         <v>0</v>
       </c>
       <c r="M16" s="12">
-        <v>2595.2089624597984</v>
+        <v>3468.3843359875855</v>
       </c>
       <c r="N16" s="12">
-        <v>129.73024600871355</v>
+        <v>173.37885298221249</v>
       </c>
       <c r="O16" s="12">
-        <v>271540.88291616889</v>
+        <v>71121.619973854409</v>
       </c>
       <c r="P16" s="12">
-        <v>125525.19314700128</v>
+        <v>444311.31590146915</v>
       </c>
       <c r="Q16" s="12">
-        <v>6264.6975631650184</v>
+        <v>22160.631367963128</v>
       </c>
       <c r="R16" s="12">
-        <v>2705988.2796105715</v>
+        <v>1283263.8094927592</v>
       </c>
       <c r="S16" s="12">
-        <v>2924804.4762411872</v>
+        <v>12328903.445420463</v>
       </c>
       <c r="T16" s="12">
-        <v>145886.35632553152</v>
+        <v>614624.27912978223</v>
       </c>
       <c r="U16" s="12">
-        <v>24174097.486484967</v>
+        <v>15709966.526057255</v>
       </c>
       <c r="V16" s="13">
-        <v>0</v>
+        <v>0.69062733711944724</v>
       </c>
       <c r="W16" s="13"/>
       <c r="X16" s="5">
@@ -2324,7 +2325,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>22</v>
       </c>
@@ -2335,61 +2336,61 @@
         <v>2.4499999999999999E-5</v>
       </c>
       <c r="D17" s="11">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E17" s="10">
         <v>0</v>
       </c>
       <c r="F17" s="12">
-        <v>8994154.4463011809</v>
+        <v>9767502.2388567403</v>
       </c>
       <c r="G17" s="12">
-        <v>4296.90464899363</v>
+        <v>4762.0873802695796</v>
       </c>
       <c r="H17" s="12">
-        <v>214.79522660925701</v>
+        <v>238.04894954270199</v>
       </c>
       <c r="I17" s="12">
-        <v>449592.03635317902</v>
+        <v>97649.895782205102</v>
       </c>
       <c r="J17" s="12">
         <v>0</v>
       </c>
       <c r="K17" s="12">
-        <v>5194884.6289435411</v>
+        <v>7162386.8502112823</v>
       </c>
       <c r="L17" s="12">
         <v>0</v>
       </c>
       <c r="M17" s="12">
-        <v>2403.4593697758864</v>
+        <v>3383.8804901305575</v>
       </c>
       <c r="N17" s="12">
-        <v>120.14499788773854</v>
+        <v>169.15464411491376</v>
       </c>
       <c r="O17" s="12">
-        <v>251477.81499008797</v>
+        <v>69388.810161223941</v>
       </c>
       <c r="P17" s="12">
-        <v>122929.98418454148</v>
+        <v>440842.93156548165</v>
       </c>
       <c r="Q17" s="12">
-        <v>6134.9673171563045</v>
+        <v>21987.252514980915</v>
       </c>
       <c r="R17" s="12">
-        <v>2434447.3966944027</v>
+        <v>1212142.1895189048</v>
       </c>
       <c r="S17" s="12">
-        <v>2799279.2830941863</v>
+        <v>11884592.129518993</v>
       </c>
       <c r="T17" s="12">
-        <v>139621.65876236651</v>
+        <v>592463.64776181907</v>
       </c>
       <c r="U17" s="12">
-        <v>21468109.206874393</v>
+        <v>14426702.716564497</v>
       </c>
       <c r="V17" s="13">
-        <v>0</v>
+        <v>0.69796246411531304</v>
       </c>
       <c r="W17" s="13"/>
       <c r="X17" s="5">
@@ -2471,7 +2472,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>23</v>
       </c>
@@ -2482,61 +2483,61 @@
         <v>2.4499999999999999E-5</v>
       </c>
       <c r="D18" s="11">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E18" s="10">
         <v>0</v>
       </c>
       <c r="F18" s="12">
-        <v>8540050.7100724</v>
+        <v>9664852.206744723</v>
       </c>
       <c r="G18" s="12">
-        <v>4079.9592466240601</v>
+        <v>4712.0409701893996</v>
       </c>
       <c r="H18" s="12">
-        <v>203.95048122382701</v>
+        <v>235.54721146092501</v>
       </c>
       <c r="I18" s="12">
-        <v>426892.69038290298</v>
+        <v>96623.659525211799</v>
       </c>
       <c r="J18" s="12">
         <v>0</v>
       </c>
       <c r="K18" s="12">
-        <v>4811055.4167109746</v>
+        <v>6987882.188753007</v>
       </c>
       <c r="L18" s="12">
         <v>0</v>
       </c>
       <c r="M18" s="12">
-        <v>2225.8773862619082</v>
+        <v>3301.4354991387513</v>
       </c>
       <c r="N18" s="12">
-        <v>111.2679653476893</v>
+        <v>165.03335403065961</v>
       </c>
       <c r="O18" s="12">
-        <v>232897.12677156192</v>
+        <v>67698.218591764147</v>
       </c>
       <c r="P18" s="12">
-        <v>120526.52481476559</v>
+        <v>437459.05107535102</v>
       </c>
       <c r="Q18" s="12">
-        <v>6014.8223192685664</v>
+        <v>21818.097870866</v>
       </c>
       <c r="R18" s="12">
-        <v>2182969.5817043139</v>
+        <v>1142753.3793576809</v>
       </c>
       <c r="S18" s="12">
-        <v>2676349.2989096446</v>
+        <v>11443749.197953513</v>
       </c>
       <c r="T18" s="12">
-        <v>133486.69144521025</v>
+        <v>570476.39524683822</v>
       </c>
       <c r="U18" s="12">
-        <v>19033661.81017999</v>
+        <v>13214560.527045595</v>
       </c>
       <c r="V18" s="13">
-        <v>0</v>
+        <v>0.70537549721937032</v>
       </c>
       <c r="W18" s="13"/>
       <c r="X18" s="5">
@@ -2618,7 +2619,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>24</v>
       </c>
@@ -2629,61 +2630,61 @@
         <v>2.5000000000000001E-5</v>
       </c>
       <c r="D19" s="11">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E19" s="10">
         <v>0</v>
       </c>
       <c r="F19" s="12">
-        <v>8108874.1099616494</v>
+        <v>9563280.9590378609</v>
       </c>
       <c r="G19" s="12">
-        <v>3953.0267151547</v>
+        <v>4757.6728054678697</v>
       </c>
       <c r="H19" s="12">
-        <v>197.60439297870801</v>
+        <v>237.827142202603</v>
       </c>
       <c r="I19" s="12">
-        <v>405337.27779240097</v>
+        <v>95607.706276713696</v>
       </c>
       <c r="J19" s="12">
         <v>0</v>
       </c>
       <c r="K19" s="12">
-        <v>4455585.8071810845</v>
+        <v>6817629.1654018983</v>
       </c>
       <c r="L19" s="12">
         <v>0</v>
       </c>
       <c r="M19" s="12">
-        <v>2103.4854170179892</v>
+        <v>3286.733056872919</v>
       </c>
       <c r="N19" s="12">
-        <v>105.14929164933247</v>
+        <v>164.29762240071528</v>
       </c>
       <c r="O19" s="12">
-        <v>215688.15852961372</v>
+        <v>66048.469821280465</v>
       </c>
       <c r="P19" s="12">
-        <v>118300.6474285037</v>
+        <v>434157.61557621224</v>
       </c>
       <c r="Q19" s="12">
-        <v>5903.5543539208766</v>
+        <v>21653.06451683534</v>
       </c>
       <c r="R19" s="12">
-        <v>1950072.4549327521</v>
+        <v>1075055.1607659163</v>
       </c>
       <c r="S19" s="12">
-        <v>2555822.7740948787</v>
+        <v>11006290.146878162</v>
       </c>
       <c r="T19" s="12">
-        <v>127471.86912594164</v>
+        <v>548658.29737597238</v>
       </c>
       <c r="U19" s="12">
-        <v>16850692.228475671</v>
+        <v>12071807.147687912</v>
       </c>
       <c r="V19" s="13">
-        <v>0</v>
+        <v>0.71286726386946653</v>
       </c>
       <c r="W19" s="13"/>
       <c r="X19" s="5">
@@ -2765,7 +2766,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>25</v>
       </c>
@@ -2776,61 +2777,61 @@
         <v>2.5999999999999998E-5</v>
       </c>
       <c r="D20" s="11">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E20" s="10">
         <v>0</v>
       </c>
       <c r="F20" s="12">
-        <v>7699386.2010611156</v>
+        <v>9462677.7528134771</v>
       </c>
       <c r="G20" s="12">
-        <v>3903.5380572835302</v>
+        <v>4895.9258214425899</v>
       </c>
       <c r="H20" s="12">
-        <v>195.12869354244799</v>
+        <v>244.73582560218401</v>
       </c>
       <c r="I20" s="12">
-        <v>384864.214732608</v>
+        <v>94600.944737708094</v>
       </c>
       <c r="J20" s="12">
         <v>0</v>
       </c>
       <c r="K20" s="12">
-        <v>4126337.075704623</v>
+        <v>6651454.3194355322</v>
       </c>
       <c r="L20" s="12">
         <v>0</v>
       </c>
       <c r="M20" s="12">
-        <v>2025.9677035013738</v>
+        <v>3334.8844678613145</v>
       </c>
       <c r="N20" s="12">
-        <v>101.27336414865717</v>
+        <v>166.70303703446527</v>
       </c>
       <c r="O20" s="12">
-        <v>199747.62839235386</v>
+        <v>64437.908734048549</v>
       </c>
       <c r="P20" s="12">
-        <v>116197.16201148571</v>
+        <v>430870.88251933939</v>
       </c>
       <c r="Q20" s="12">
-        <v>5798.405062271544</v>
+        <v>21488.766894434626</v>
       </c>
       <c r="R20" s="12">
-        <v>1734384.2964031384</v>
+        <v>1009006.6909446355</v>
       </c>
       <c r="S20" s="12">
-        <v>2437522.1266663745</v>
+        <v>10572132.531301951</v>
       </c>
       <c r="T20" s="12">
-        <v>121568.31477202076</v>
+        <v>527005.232859137</v>
       </c>
       <c r="U20" s="12">
-        <v>14900619.77354292</v>
+        <v>10996751.986921996</v>
       </c>
       <c r="V20" s="13">
-        <v>0</v>
+        <v>0.72044616851264209</v>
       </c>
       <c r="W20" s="13"/>
       <c r="X20" s="5">
@@ -2912,7 +2913,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
         <v>26</v>
       </c>
@@ -2923,61 +2924,61 @@
         <v>2.7500000000000004E-5</v>
       </c>
       <c r="D21" s="11">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="E21" s="10">
         <v>0</v>
       </c>
       <c r="F21" s="12">
-        <v>7310423.3195776818</v>
+        <v>9362936.1464287248</v>
       </c>
       <c r="G21" s="12">
-        <v>3940.2639898775401</v>
+        <v>5123.7963529645403</v>
       </c>
       <c r="H21" s="12">
-        <v>196.96172908779101</v>
+        <v>256.12288713807197</v>
       </c>
       <c r="I21" s="12">
-        <v>292332.49849946803</v>
+        <v>93602.326340200496</v>
       </c>
       <c r="J21" s="12">
         <v>0</v>
       </c>
       <c r="K21" s="12">
-        <v>3821338.1290680766</v>
+        <v>6489193.5258915285</v>
       </c>
       <c r="L21" s="12">
         <v>0</v>
       </c>
       <c r="M21" s="12">
-        <v>1994.6365075434428</v>
+        <v>3441.231792680489</v>
       </c>
       <c r="N21" s="12">
-        <v>99.705770079531931</v>
+        <v>172.01663792564662</v>
       </c>
       <c r="O21" s="12">
-        <v>147984.26586299608</v>
+        <v>62864.969464367285</v>
       </c>
       <c r="P21" s="12">
-        <v>114171.19430798433</v>
+        <v>427535.998051478</v>
       </c>
       <c r="Q21" s="12">
-        <v>5697.1316981228865</v>
+        <v>21322.06385740016</v>
       </c>
       <c r="R21" s="12">
-        <v>1534636.6680107843</v>
+        <v>944568.78221058706</v>
       </c>
       <c r="S21" s="12">
-        <v>2321324.964654888</v>
+        <v>10141261.648782611</v>
       </c>
       <c r="T21" s="12">
-        <v>115769.9097097492</v>
+        <v>505516.46596470242</v>
       </c>
       <c r="U21" s="12">
-        <v>13166235.477139784</v>
+        <v>9987745.2959773615</v>
       </c>
       <c r="V21" s="13">
-        <v>0</v>
+        <v>0.72812094670586935</v>
       </c>
       <c r="W21" s="13"/>
       <c r="X21" s="5">
@@ -3059,7 +3060,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>27</v>
       </c>
@@ -3070,61 +3071,61 @@
         <v>2.9999999999999997E-5</v>
       </c>
       <c r="D22" s="11">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="E22" s="10">
         <v>0</v>
       </c>
       <c r="F22" s="12">
-        <v>7013953.5953592481</v>
+        <v>9263953.9008484222</v>
       </c>
       <c r="G22" s="12">
-        <v>4124.1428510005298</v>
+        <v>5530.4975200993304</v>
       </c>
       <c r="H22" s="12">
-        <v>206.14837263285099</v>
+        <v>276.44606523314297</v>
       </c>
       <c r="I22" s="12">
-        <v>280469.76926158002</v>
+        <v>92610.357970574507</v>
       </c>
       <c r="J22" s="12">
         <v>0</v>
       </c>
       <c r="K22" s="12">
-        <v>3576021.9327523056</v>
+        <v>6330691.5275922706</v>
       </c>
       <c r="L22" s="12">
         <v>0</v>
       </c>
       <c r="M22" s="12">
-        <v>2036.2752737081939</v>
+        <v>3662.3712894175719</v>
       </c>
       <c r="N22" s="12">
-        <v>101.78474632749901</v>
+        <v>183.06637489716044</v>
       </c>
       <c r="O22" s="12">
-        <v>138480.57082490341</v>
+        <v>61327.848878236931</v>
       </c>
       <c r="P22" s="12">
-        <v>112176.55780044087</v>
+        <v>424094.76625879755</v>
       </c>
       <c r="Q22" s="12">
-        <v>5597.4259280433535</v>
+        <v>21150.047219474516</v>
       </c>
       <c r="R22" s="12">
-        <v>1386652.4021477881</v>
+        <v>881703.8127462198</v>
       </c>
       <c r="S22" s="12">
-        <v>2207153.7703469042</v>
+        <v>9713725.6507311314</v>
       </c>
       <c r="T22" s="12">
-        <v>110072.77801162632</v>
+        <v>484194.40210730222</v>
       </c>
       <c r="U22" s="12">
-        <v>11631598.809128998</v>
+        <v>9043176.5137667749</v>
       </c>
       <c r="V22" s="13">
-        <v>0</v>
+        <v>0.73590067522463953</v>
       </c>
       <c r="W22" s="13"/>
       <c r="X22" s="5">
@@ -3206,7 +3207,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
         <v>28</v>
       </c>
@@ -3217,61 +3218,61 @@
         <v>3.2499999999999997E-5</v>
       </c>
       <c r="D23" s="11">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="E23" s="10">
         <v>0</v>
       </c>
       <c r="F23" s="12">
-        <v>6729153.534874035</v>
+        <v>9165536.5992925148</v>
       </c>
       <c r="G23" s="12">
-        <v>4286.4011465642297</v>
+        <v>5927.7144686669999</v>
       </c>
       <c r="H23" s="12">
-        <v>214.25388493521001</v>
+        <v>296.29421285419301</v>
       </c>
       <c r="I23" s="12">
-        <v>269074.28987074399</v>
+        <v>91624.089083334999</v>
       </c>
       <c r="J23" s="12">
         <v>0</v>
       </c>
       <c r="K23" s="12">
-        <v>3346278.3753738431</v>
+        <v>6175736.6120361099</v>
       </c>
       <c r="L23" s="12">
         <v>0</v>
       </c>
       <c r="M23" s="12">
-        <v>2064.238834587482</v>
+        <v>3870.450765384825</v>
       </c>
       <c r="N23" s="12">
-        <v>103.18007452452308</v>
+        <v>193.46278721459598</v>
       </c>
       <c r="O23" s="12">
-        <v>129580.40546098851</v>
+        <v>59825.169986642133</v>
       </c>
       <c r="P23" s="12">
-        <v>110140.28252673268</v>
+        <v>420432.39496937994</v>
       </c>
       <c r="Q23" s="12">
-        <v>5495.6411817158551</v>
+        <v>20966.980844577352</v>
       </c>
       <c r="R23" s="12">
-        <v>1248171.8313228851</v>
+        <v>820375.96386798285</v>
       </c>
       <c r="S23" s="12">
-        <v>2094977.2125464638</v>
+        <v>9289630.8844723348</v>
       </c>
       <c r="T23" s="12">
-        <v>104475.35208358297</v>
+        <v>463044.35488782765</v>
       </c>
       <c r="U23" s="12">
-        <v>10244946.406981207</v>
+        <v>8161472.7010205528</v>
       </c>
       <c r="V23" s="13">
-        <v>0</v>
+        <v>0.74380259759265122</v>
       </c>
       <c r="W23" s="13"/>
       <c r="X23" s="5">
@@ -3353,7 +3354,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A24" s="8">
         <v>29</v>
       </c>
@@ -3364,61 +3365,61 @@
         <v>3.5000000000000004E-5</v>
       </c>
       <c r="D24" s="11">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="E24" s="10">
         <v>0</v>
       </c>
       <c r="F24" s="12">
-        <v>6455578.589971792</v>
+        <v>9067688.5015276596</v>
       </c>
       <c r="G24" s="12">
-        <v>4428.4494134996803</v>
+        <v>6315.5345175257899</v>
       </c>
       <c r="H24" s="12">
-        <v>221.34884641506</v>
+        <v>315.671728277478</v>
       </c>
       <c r="I24" s="12">
-        <v>258128.24817521599</v>
+        <v>90643.561815429406</v>
       </c>
       <c r="J24" s="12">
         <v>0</v>
       </c>
       <c r="K24" s="12">
-        <v>3131130.336434382</v>
+        <v>6024258.0225100275</v>
       </c>
       <c r="L24" s="12">
         <v>0</v>
       </c>
       <c r="M24" s="12">
-        <v>2080.0949695980185</v>
+        <v>4065.9355187646534</v>
       </c>
       <c r="N24" s="12">
-        <v>103.97016629584311</v>
+        <v>203.22917857727964</v>
       </c>
       <c r="O24" s="12">
-        <v>121245.88550196258</v>
+        <v>58356.24467097038</v>
       </c>
       <c r="P24" s="12">
-        <v>108076.04369214521</v>
+        <v>416561.94420399511</v>
       </c>
       <c r="Q24" s="12">
-        <v>5392.4611071913314</v>
+        <v>20773.518057362759</v>
       </c>
       <c r="R24" s="12">
-        <v>1118591.4258618965</v>
+        <v>760550.79388134077</v>
       </c>
       <c r="S24" s="12">
-        <v>1984836.9300197309</v>
+        <v>8869198.4895029552</v>
       </c>
       <c r="T24" s="12">
-        <v>98979.710901867133</v>
+        <v>442077.37404325034</v>
       </c>
       <c r="U24" s="12">
-        <v>8996774.5756583232</v>
+        <v>7341096.7371525699</v>
       </c>
       <c r="V24" s="13">
-        <v>0</v>
+        <v>0.75182886242020219</v>
       </c>
       <c r="W24" s="13"/>
       <c r="X24" s="5">
@@ -3500,7 +3501,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A25" s="8">
         <v>30</v>
       </c>
@@ -3511,61 +3512,61 @@
         <v>3.7500000000000003E-5</v>
       </c>
       <c r="D25" s="11">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="E25" s="10">
         <v>0</v>
       </c>
       <c r="F25" s="12">
-        <v>6192800.5435366612</v>
+        <v>8970413.7334664259</v>
       </c>
       <c r="G25" s="12">
-        <v>4551.6230549669599</v>
+        <v>6694.0457328884104</v>
       </c>
       <c r="H25" s="12">
-        <v>227.500075442482</v>
+        <v>334.58304671905501</v>
       </c>
       <c r="I25" s="12">
-        <v>247614.48687463099</v>
+        <v>89668.816961321005</v>
       </c>
       <c r="J25" s="12">
         <v>0</v>
       </c>
       <c r="K25" s="12">
-        <v>2929661.2705691447</v>
+        <v>5876186.1960329646</v>
       </c>
       <c r="L25" s="12">
         <v>0</v>
       </c>
       <c r="M25" s="12">
-        <v>2085.2691015535288</v>
+        <v>4249.2780641945028</v>
       </c>
       <c r="N25" s="12">
-        <v>104.2263105253447</v>
+        <v>212.38821152498767</v>
       </c>
       <c r="O25" s="12">
-        <v>113441.47622533033</v>
+        <v>56920.396447844978</v>
       </c>
       <c r="P25" s="12">
-        <v>105995.94872254718</v>
+        <v>412496.00868523045</v>
       </c>
       <c r="Q25" s="12">
-        <v>5288.4909408954891</v>
+        <v>20570.288878785479</v>
       </c>
       <c r="R25" s="12">
-        <v>997345.54035993409</v>
+        <v>702194.5492103704</v>
       </c>
       <c r="S25" s="12">
-        <v>1876760.8863275854</v>
+        <v>8452636.5452989601</v>
       </c>
       <c r="T25" s="12">
-        <v>93587.249794675809</v>
+        <v>421303.85598588758</v>
       </c>
       <c r="U25" s="12">
-        <v>7878183.1497964263</v>
+        <v>6580545.9432712281</v>
       </c>
       <c r="V25" s="13">
-        <v>0</v>
+        <v>0.7599816612081578</v>
       </c>
       <c r="W25" s="13"/>
       <c r="X25" s="5">
@@ -3647,7 +3648,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A26" s="8">
         <v>31</v>
       </c>
@@ -3658,61 +3659,61 @@
         <v>4.0500000000000002E-5</v>
       </c>
       <c r="D26" s="11">
-        <v>0.04</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="E26" s="10">
         <v>0</v>
       </c>
       <c r="F26" s="12">
-        <v>5940406.9335316205</v>
+        <v>8873716.287725497</v>
       </c>
       <c r="G26" s="12">
-        <v>4715.3995350631703</v>
+        <v>7155.2206010375703</v>
       </c>
       <c r="H26" s="12">
-        <v>235.67926241763701</v>
+        <v>357.62337870812701</v>
       </c>
       <c r="I26" s="12">
-        <v>237515.23296807599</v>
+        <v>79829.485313847399</v>
       </c>
       <c r="J26" s="12">
         <v>0</v>
       </c>
       <c r="K26" s="12">
-        <v>2741011.499072541</v>
+        <v>5731452.7484621713</v>
       </c>
       <c r="L26" s="12">
         <v>0</v>
       </c>
       <c r="M26" s="12">
-        <v>2107.0685253719053</v>
+        <v>4478.4281062133796</v>
       </c>
       <c r="N26" s="12">
-        <v>105.31289071699329</v>
+        <v>223.83524980532718</v>
       </c>
       <c r="O26" s="12">
-        <v>106133.29113727028</v>
+        <v>49965.001873211324</v>
       </c>
       <c r="P26" s="12">
-        <v>103910.67962099364</v>
+        <v>408246.73062103597</v>
       </c>
       <c r="Q26" s="12">
-        <v>5184.2646303701449</v>
+        <v>20357.900667260492</v>
       </c>
       <c r="R26" s="12">
-        <v>883904.06413460383</v>
+        <v>645274.15276252537</v>
       </c>
       <c r="S26" s="12">
-        <v>1770764.9376050385</v>
+        <v>8040140.5366137289</v>
       </c>
       <c r="T26" s="12">
-        <v>88298.758853780324</v>
+        <v>400733.56710710214</v>
       </c>
       <c r="U26" s="12">
-        <v>6880837.6094364924</v>
+        <v>5878351.3940608585</v>
       </c>
       <c r="V26" s="13">
-        <v>0</v>
+        <v>0.76826322927569102</v>
       </c>
       <c r="W26" s="13"/>
       <c r="X26" s="5">
@@ -3794,7 +3795,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A27" s="8">
         <v>32</v>
       </c>
@@ -3805,61 +3806,61 @@
         <v>4.35E-5</v>
       </c>
       <c r="D27" s="11">
-        <v>0.03</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="E27" s="10">
         <v>0</v>
       </c>
       <c r="F27" s="12">
-        <v>5697940.6217660643</v>
+        <v>8786373.9584319033</v>
       </c>
       <c r="G27" s="12">
-        <v>4882.74401383023</v>
+        <v>7609.5811777979898</v>
       </c>
       <c r="H27" s="12">
-        <v>244.036308798927</v>
+        <v>380.32182249892202</v>
       </c>
       <c r="I27" s="12">
-        <v>170860.144238901</v>
+        <v>79041.247787308195</v>
       </c>
       <c r="J27" s="12">
         <v>0</v>
       </c>
       <c r="K27" s="12">
-        <v>2564347.7790330481</v>
+        <v>5595578.1155629568</v>
       </c>
       <c r="L27" s="12">
         <v>0</v>
       </c>
       <c r="M27" s="12">
-        <v>2128.0825160308077</v>
+        <v>4696.1227004890952</v>
       </c>
       <c r="N27" s="12">
-        <v>106.36015334015183</v>
+        <v>234.70909927862866</v>
       </c>
       <c r="O27" s="12">
-        <v>74467.243134476856</v>
+        <v>48778.952393852145</v>
       </c>
       <c r="P27" s="12">
-        <v>101803.61109562175</v>
+        <v>403768.30251482263</v>
       </c>
       <c r="Q27" s="12">
-        <v>5078.951739653151</v>
+        <v>20134.065417455164</v>
       </c>
       <c r="R27" s="12">
-        <v>777770.77299733344</v>
+        <v>595309.15088931401</v>
       </c>
       <c r="S27" s="12">
-        <v>1666854.2579840447</v>
+        <v>7631893.8059926927</v>
       </c>
       <c r="T27" s="12">
-        <v>83114.494223410176</v>
+        <v>380375.66643984162</v>
       </c>
       <c r="U27" s="12">
-        <v>5996933.5453018891</v>
+        <v>5233077.2412983328</v>
       </c>
       <c r="V27" s="13">
-        <v>0</v>
+        <v>0.77590027047983445</v>
       </c>
       <c r="W27" s="13"/>
       <c r="X27" s="5">
@@ -3941,7 +3942,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A28" s="8">
         <v>33</v>
       </c>
@@ -3952,61 +3953,61 @@
         <v>4.6500000000000005E-5</v>
       </c>
       <c r="D28" s="11">
-        <v>0.03</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="E28" s="10">
         <v>0</v>
       </c>
       <c r="F28" s="12">
-        <v>5521953.697204534</v>
+        <v>8699342.8076443002</v>
       </c>
       <c r="G28" s="12">
-        <v>5058.2680768570499</v>
+        <v>8053.7948063762797</v>
       </c>
       <c r="H28" s="12">
-        <v>252.80167674904999</v>
+        <v>402.51184799003101</v>
       </c>
       <c r="I28" s="12">
-        <v>165577.72989033299</v>
+        <v>78255.859028123101</v>
       </c>
       <c r="J28" s="12">
         <v>0</v>
       </c>
       <c r="K28" s="12">
-        <v>2423907.8749783915</v>
+        <v>5462580.2112542726</v>
       </c>
       <c r="L28" s="12">
         <v>0</v>
       </c>
       <c r="M28" s="12">
-        <v>2150.2586011839244</v>
+        <v>4900.6687042753038</v>
       </c>
       <c r="N28" s="12">
-        <v>107.4654351180852</v>
+        <v>244.92518917703885</v>
       </c>
       <c r="O28" s="12">
-        <v>70386.727720136783</v>
+        <v>47618.054406064177</v>
       </c>
       <c r="P28" s="12">
-        <v>99675.528579590929</v>
+        <v>399072.1798143335</v>
       </c>
       <c r="Q28" s="12">
-        <v>4972.5915863129994</v>
+        <v>19899.356318176538</v>
       </c>
       <c r="R28" s="12">
-        <v>703303.52986285673</v>
+        <v>546530.19849546195</v>
       </c>
       <c r="S28" s="12">
-        <v>1565050.646888423</v>
+        <v>7228125.5034778696</v>
       </c>
       <c r="T28" s="12">
-        <v>78035.542483757032</v>
+        <v>360241.60102238646</v>
       </c>
       <c r="U28" s="12">
-        <v>5219162.7723045554</v>
+        <v>4637768.09040902</v>
       </c>
       <c r="V28" s="13">
-        <v>0</v>
+        <v>0.78366263769876221</v>
       </c>
       <c r="W28" s="13"/>
       <c r="X28" s="5">
@@ -4088,7 +4089,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A29" s="8">
         <v>34</v>
       </c>
@@ -4099,61 +4100,61 @@
         <v>4.9500000000000004E-5</v>
       </c>
       <c r="D29" s="11">
-        <v>0.03</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="E29" s="10">
         <v>0</v>
       </c>
       <c r="F29" s="12">
-        <v>5351064.8975605955</v>
+        <v>8612630.6419618111</v>
       </c>
       <c r="G29" s="12">
-        <v>5217.9617871055798</v>
+        <v>8487.9249846893708</v>
       </c>
       <c r="H29" s="12">
-        <v>260.775398992173</v>
+        <v>424.19667195872802</v>
       </c>
       <c r="I29" s="12">
-        <v>160448.51241411999</v>
+        <v>77473.388994310299</v>
       </c>
       <c r="J29" s="12">
         <v>0</v>
       </c>
       <c r="K29" s="12">
-        <v>2291014.8858297123</v>
+        <v>5332407.2123937244</v>
       </c>
       <c r="L29" s="12">
         <v>0</v>
       </c>
       <c r="M29" s="12">
-        <v>2163.4860014470587</v>
+        <v>5092.5161962777038</v>
       </c>
       <c r="N29" s="12">
-        <v>108.1234298487058</v>
+        <v>254.50606906323637</v>
       </c>
       <c r="O29" s="12">
-        <v>66525.613778690837</v>
+        <v>46481.853803575599</v>
       </c>
       <c r="P29" s="12">
-        <v>97525.269978407014</v>
+        <v>394171.51111005823</v>
       </c>
       <c r="Q29" s="12">
-        <v>4865.1261511949142</v>
+        <v>19654.431128999498</v>
       </c>
       <c r="R29" s="12">
-        <v>632916.80214272009</v>
+        <v>498912.1440893978</v>
       </c>
       <c r="S29" s="12">
-        <v>1465375.1183088326</v>
+        <v>6829053.3236635365</v>
       </c>
       <c r="T29" s="12">
-        <v>73062.95089744404</v>
+        <v>340342.24470420991</v>
       </c>
       <c r="U29" s="12">
-        <v>4515859.242441698</v>
+        <v>4091237.8919135593</v>
       </c>
       <c r="V29" s="13">
-        <v>0</v>
+        <v>0.79155257136760382</v>
       </c>
       <c r="W29" s="13"/>
       <c r="X29" s="5">
@@ -4235,7 +4236,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A30" s="8">
         <v>35</v>
       </c>
@@ -4246,61 +4247,61 @@
         <v>5.3499999999999999E-5</v>
       </c>
       <c r="D30" s="11">
-        <v>0.03</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="E30" s="10">
         <v>0</v>
       </c>
       <c r="F30" s="12">
-        <v>5185137.6479603779</v>
+        <v>8526245.1313108522</v>
       </c>
       <c r="G30" s="12">
-        <v>5464.7296386395501</v>
+        <v>9081.7854759351103</v>
       </c>
       <c r="H30" s="12">
-        <v>273.09760577509797</v>
+        <v>453.85847674952697</v>
       </c>
       <c r="I30" s="12">
-        <v>155466.74913277299</v>
+        <v>76693.100716166096</v>
       </c>
       <c r="J30" s="12">
         <v>0</v>
       </c>
       <c r="K30" s="12">
-        <v>2165271.3361619799</v>
+        <v>5205008.0026124464</v>
       </c>
       <c r="L30" s="12">
         <v>0</v>
       </c>
       <c r="M30" s="12">
-        <v>2209.9691932309966</v>
+        <v>5372.522312077529</v>
       </c>
       <c r="N30" s="12">
-        <v>110.44229731708397</v>
+        <v>268.4895827283662</v>
       </c>
       <c r="O30" s="12">
-        <v>62871.67872420745</v>
+        <v>45369.426075062198</v>
       </c>
       <c r="P30" s="12">
-        <v>95361.783976959952</v>
+        <v>389078.99491378054</v>
       </c>
       <c r="Q30" s="12">
-        <v>4757.002721346209</v>
+        <v>19399.92505993626</v>
       </c>
       <c r="R30" s="12">
-        <v>566391.18836402928</v>
+        <v>452430.29028582218</v>
       </c>
       <c r="S30" s="12">
-        <v>1367849.8483304258</v>
+        <v>6434881.8125534784</v>
       </c>
       <c r="T30" s="12">
-        <v>68197.824746249127</v>
+        <v>320687.8135752104</v>
       </c>
       <c r="U30" s="12">
-        <v>3882942.4402989792</v>
+        <v>3592325.7478241613</v>
       </c>
       <c r="V30" s="13">
-        <v>0</v>
+        <v>0.79957235874546884</v>
       </c>
       <c r="W30" s="13"/>
       <c r="X30" s="5">
@@ -4382,7 +4383,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A31" s="8">
         <v>36</v>
       </c>
@@ -4393,61 +4394,61 @@
         <v>5.8E-5</v>
       </c>
       <c r="D31" s="11">
-        <v>0.03</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="E31" s="10">
         <v>0</v>
       </c>
       <c r="F31" s="12">
-        <v>5023933.07158319</v>
+        <v>8440016.3866420016</v>
       </c>
       <c r="G31" s="12">
-        <v>5740.1794575590502</v>
+        <v>9755.86961355124</v>
       </c>
       <c r="H31" s="12">
-        <v>286.85082634764802</v>
+        <v>487.524698675031</v>
       </c>
       <c r="I31" s="12">
-        <v>150626.20742535399</v>
+        <v>59044.135910365301</v>
       </c>
       <c r="J31" s="12">
         <v>0</v>
       </c>
       <c r="K31" s="12">
-        <v>2046257.2250348877</v>
+        <v>5080225.3742360836</v>
       </c>
       <c r="L31" s="12">
         <v>0</v>
       </c>
       <c r="M31" s="12">
-        <v>2264.1612488163423</v>
+        <v>5690.4823230259653</v>
       </c>
       <c r="N31" s="12">
-        <v>113.14568298940839</v>
+        <v>284.36733881675644</v>
       </c>
       <c r="O31" s="12">
-        <v>59413.128880413671</v>
+        <v>34439.739867943208</v>
       </c>
       <c r="P31" s="12">
-        <v>93151.814783728958</v>
+        <v>383706.47260170296</v>
       </c>
       <c r="Q31" s="12">
-        <v>4646.560424029125</v>
+        <v>19131.435477207895</v>
       </c>
       <c r="R31" s="12">
-        <v>503519.50963982177</v>
+        <v>407060.86421075993</v>
       </c>
       <c r="S31" s="12">
-        <v>1272488.0643534653</v>
+        <v>6045802.8176396992</v>
       </c>
       <c r="T31" s="12">
-        <v>63440.822024902918</v>
+        <v>301287.88851527416</v>
       </c>
       <c r="U31" s="12">
-        <v>3316551.2519349493</v>
+        <v>3139895.4575383388</v>
       </c>
       <c r="V31" s="13">
-        <v>0</v>
+        <v>0.80774131453987397</v>
       </c>
       <c r="W31" s="13"/>
       <c r="X31" s="5">
@@ -4529,7 +4530,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A32" s="8">
         <v>37</v>
       </c>
@@ -4540,61 +4541,61 @@
         <v>6.3500000000000012E-5</v>
       </c>
       <c r="D32" s="11">
-        <v>0.03</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="E32" s="10">
         <v>0</v>
       </c>
       <c r="F32" s="12">
-        <v>4867279.8338739295</v>
+        <v>8370728.8564194106</v>
       </c>
       <c r="G32" s="12">
-        <v>6088.5303912068603</v>
+        <v>10593.2814105221</v>
       </c>
       <c r="H32" s="12">
-        <v>304.24286843149503</v>
+        <v>529.34454053048103</v>
       </c>
       <c r="I32" s="12">
-        <v>145921.040195254</v>
+        <v>58556.034892031203</v>
       </c>
       <c r="J32" s="12">
         <v>0</v>
       </c>
       <c r="K32" s="12">
-        <v>1933601.7943838029</v>
+        <v>4967971.1659860546</v>
       </c>
       <c r="L32" s="12">
         <v>0</v>
       </c>
       <c r="M32" s="12">
-        <v>2342.3873021395179</v>
+        <v>6092.4181486560719</v>
       </c>
       <c r="N32" s="12">
-        <v>117.04871060669477</v>
+        <v>304.43713903574712</v>
       </c>
       <c r="O32" s="12">
-        <v>56138.931680786314</v>
+        <v>33676.802858762763</v>
       </c>
       <c r="P32" s="12">
-        <v>90887.653534912606</v>
+        <v>378015.99027867703</v>
       </c>
       <c r="Q32" s="12">
-        <v>4533.4147410397163</v>
+        <v>18847.06813839114</v>
       </c>
       <c r="R32" s="12">
-        <v>444106.38075940806</v>
+        <v>372621.12434281677</v>
       </c>
       <c r="S32" s="12">
-        <v>1179336.2495697367</v>
+        <v>5662096.3450379968</v>
       </c>
       <c r="T32" s="12">
-        <v>58794.26160087379</v>
+        <v>282156.45303806622</v>
       </c>
       <c r="U32" s="12">
-        <v>2813031.7422951283</v>
+        <v>2732834.5933275786</v>
       </c>
       <c r="V32" s="13">
-        <v>0</v>
+        <v>0.81442727960972539</v>
       </c>
       <c r="W32" s="13"/>
       <c r="X32" s="5">
@@ -4676,7 +4677,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
         <v>38</v>
       </c>
@@ -4687,61 +4688,61 @@
         <v>6.9499999999999995E-5</v>
       </c>
       <c r="D33" s="11">
-        <v>0.03</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="E33" s="10">
         <v>0</v>
       </c>
       <c r="F33" s="12">
-        <v>4714966.020419037</v>
+        <v>8301050.1955763269</v>
       </c>
       <c r="G33" s="12">
-        <v>6455.2713983802196</v>
+        <v>11497.675604537701</v>
       </c>
       <c r="H33" s="12">
-        <v>322.55045786632797</v>
+        <v>574.50420002057899</v>
       </c>
       <c r="I33" s="12">
-        <v>141345.761635139</v>
+        <v>58064.948932737898</v>
       </c>
       <c r="J33" s="12">
         <v>0</v>
       </c>
       <c r="K33" s="12">
-        <v>1826937.2706924726</v>
+        <v>4857635.6200214876</v>
       </c>
       <c r="L33" s="12">
         <v>0</v>
       </c>
       <c r="M33" s="12">
-        <v>2422.2840909503529</v>
+        <v>6519.9662474761199</v>
       </c>
       <c r="N33" s="12">
-        <v>121.03423611506206</v>
+        <v>325.78306450819838</v>
       </c>
       <c r="O33" s="12">
-        <v>53038.759891329908</v>
+        <v>32926.786267431627</v>
       </c>
       <c r="P33" s="12">
-        <v>88545.266232773094</v>
+        <v>371923.572130021</v>
       </c>
       <c r="Q33" s="12">
-        <v>4416.3660304330224</v>
+        <v>18542.630999355391</v>
       </c>
       <c r="R33" s="12">
-        <v>387967.44907862169</v>
+        <v>338944.32148405397</v>
       </c>
       <c r="S33" s="12">
-        <v>1088448.5960348241</v>
+        <v>5284080.3547593197</v>
       </c>
       <c r="T33" s="12">
-        <v>54260.846859834077</v>
+        <v>263309.38489967503</v>
       </c>
       <c r="U33" s="12">
-        <v>2368925.3615357205</v>
+        <v>2360213.4689847622</v>
       </c>
       <c r="V33" s="13">
-        <v>0</v>
+        <v>0.82126354741443308</v>
       </c>
       <c r="W33" s="13"/>
       <c r="X33" s="5">
@@ -4823,7 +4824,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A34" s="8">
         <v>39</v>
       </c>
@@ -4834,61 +4835,61 @@
         <v>7.75E-5</v>
       </c>
       <c r="D34" s="11">
-        <v>0.03</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="E34" s="10">
         <v>0</v>
       </c>
       <c r="F34" s="12">
-        <v>4566842.436927652</v>
+        <v>8230913.06683903</v>
       </c>
       <c r="G34" s="12">
-        <v>6972.1565090450304</v>
+        <v>12712.7699112891</v>
       </c>
       <c r="H34" s="12">
-        <v>348.35115299470499</v>
+        <v>635.17048858682404</v>
       </c>
       <c r="I34" s="12">
-        <v>136893.789181278</v>
+        <v>57569.5078596085</v>
       </c>
       <c r="J34" s="12">
         <v>0</v>
       </c>
       <c r="K34" s="12">
-        <v>1725938.9926094543</v>
+        <v>4749151.3662208887</v>
       </c>
       <c r="L34" s="12">
         <v>0</v>
       </c>
       <c r="M34" s="12">
-        <v>2551.7730253656196</v>
+        <v>7108.0681891690429</v>
       </c>
       <c r="N34" s="12">
-        <v>127.49471048357945</v>
+        <v>355.14173355829655</v>
       </c>
       <c r="O34" s="12">
-        <v>50102.414958656649</v>
+        <v>32188.735447781411</v>
       </c>
       <c r="P34" s="12">
-        <v>86122.982141822737</v>
+        <v>365403.60588254483</v>
       </c>
       <c r="Q34" s="12">
-        <v>4295.33179431796</v>
+        <v>18216.847934847196</v>
       </c>
       <c r="R34" s="12">
-        <v>334928.68918729178</v>
+        <v>306017.53521662235</v>
       </c>
       <c r="S34" s="12">
-        <v>999903.32980205119</v>
+        <v>4912156.782629298</v>
       </c>
       <c r="T34" s="12">
-        <v>49844.480829401051</v>
+        <v>244766.7539003196</v>
       </c>
       <c r="U34" s="12">
-        <v>1980957.9124570985</v>
+        <v>2021269.1475007078</v>
       </c>
       <c r="V34" s="13">
-        <v>0</v>
+        <v>0.82826168561423019</v>
       </c>
       <c r="W34" s="13"/>
       <c r="X34" s="5">
@@ -4970,7 +4971,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A35" s="8">
         <v>40</v>
       </c>
@@ -4981,61 +4982,61 @@
         <v>8.6500000000000002E-5</v>
       </c>
       <c r="D35" s="11">
-        <v>0.02</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="E35" s="10">
         <v>0</v>
       </c>
       <c r="F35" s="12">
-        <v>4422628.1400843346</v>
+        <v>8159995.618579546</v>
       </c>
       <c r="G35" s="12">
-        <v>7574.3076125493699</v>
+        <v>14066.775232329401</v>
       </c>
       <c r="H35" s="12">
-        <v>378.40415780305102</v>
+        <v>702.76076799088696</v>
       </c>
       <c r="I35" s="12">
-        <v>88372.229070643007</v>
+        <v>57068.092254842202</v>
       </c>
       <c r="J35" s="12">
         <v>0</v>
       </c>
       <c r="K35" s="12">
-        <v>1630249.89630641</v>
+        <v>4642308.7921310291</v>
       </c>
       <c r="L35" s="12">
         <v>0</v>
       </c>
       <c r="M35" s="12">
-        <v>2703.8475272387468</v>
+        <v>7755.0044123162106</v>
       </c>
       <c r="N35" s="12">
-        <v>135.08127722162419</v>
+        <v>387.43157309051378</v>
       </c>
       <c r="O35" s="12">
-        <v>31546.782263416651</v>
+        <v>31461.603667458556</v>
       </c>
       <c r="P35" s="12">
-        <v>83571.209116457132</v>
+        <v>358295.53769337578</v>
       </c>
       <c r="Q35" s="12">
-        <v>4167.8370838343808</v>
+        <v>17861.7062012889</v>
       </c>
       <c r="R35" s="12">
-        <v>284826.27422863513</v>
+        <v>273828.79976884089</v>
       </c>
       <c r="S35" s="12">
-        <v>913780.34766022849</v>
+        <v>4546753.176746754</v>
       </c>
       <c r="T35" s="12">
-        <v>45549.149035083086</v>
+        <v>226549.90596547243</v>
       </c>
       <c r="U35" s="12">
-        <v>1646029.2232698065</v>
+        <v>1715251.6122840857</v>
       </c>
       <c r="V35" s="13">
-        <v>0</v>
+        <v>0.8354599989443402</v>
       </c>
       <c r="W35" s="13"/>
       <c r="X35" s="5">
@@ -5117,7 +5118,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A36" s="8">
         <v>41</v>
       </c>
@@ -5128,61 +5129,61 @@
         <v>9.6500000000000015E-5</v>
       </c>
       <c r="D36" s="11">
-        <v>0.02</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E36" s="10">
         <v>0</v>
       </c>
       <c r="F36" s="12">
-        <v>4326303.1992433388</v>
+        <v>8088157.9903243836</v>
       </c>
       <c r="G36" s="12">
-        <v>8265.8686753862694</v>
+        <v>15562.563556638101</v>
       </c>
       <c r="H36" s="12">
-        <v>412.91452873173802</v>
+        <v>777.41479440412797</v>
       </c>
       <c r="I36" s="12">
-        <v>86438.395479295796</v>
+        <v>48479.778245012603</v>
       </c>
       <c r="J36" s="12">
         <v>0</v>
       </c>
       <c r="K36" s="12">
-        <v>1555446.4103228319</v>
+        <v>4537010.9550303435</v>
       </c>
       <c r="L36" s="12">
         <v>0</v>
       </c>
       <c r="M36" s="12">
-        <v>2878.0087082316718</v>
+        <v>8459.5009148502395</v>
       </c>
       <c r="N36" s="12">
-        <v>143.76850832193816</v>
+        <v>422.5872646588906</v>
       </c>
       <c r="O36" s="12">
-        <v>30096.105404597569</v>
+        <v>26352.646009949261</v>
       </c>
       <c r="P36" s="12">
-        <v>80867.361589218388</v>
+        <v>350540.53328105964</v>
       </c>
       <c r="Q36" s="12">
-        <v>4032.7558066127572</v>
+        <v>17474.274628198385</v>
       </c>
       <c r="R36" s="12">
-        <v>253279.49196521853</v>
+        <v>242367.19610138235</v>
       </c>
       <c r="S36" s="12">
-        <v>830209.13854377146</v>
+        <v>4188457.6390533783</v>
       </c>
       <c r="T36" s="12">
-        <v>41381.311951248717</v>
+        <v>208688.19976418352</v>
       </c>
       <c r="U36" s="12">
-        <v>1361202.9490411715</v>
+        <v>1441422.8125152448</v>
       </c>
       <c r="V36" s="13">
-        <v>0</v>
+        <v>0.84288041097115995</v>
       </c>
       <c r="W36" s="13"/>
       <c r="X36" s="5">
@@ -5264,7 +5265,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A37" s="8">
         <v>42</v>
       </c>
@@ -5275,61 +5276,61 @@
         <v>1.0800000000000001E-4</v>
       </c>
       <c r="D37" s="11">
-        <v>0.02</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E37" s="10">
         <v>0</v>
       </c>
       <c r="F37" s="12">
-        <v>4231186.0205599247</v>
+        <v>8023338.2337283287</v>
       </c>
       <c r="G37" s="12">
-        <v>9047.4795960832798</v>
+        <v>17277.486318453601</v>
       </c>
       <c r="H37" s="12">
-        <v>451.90981903620298</v>
+        <v>862.98793300986404</v>
       </c>
       <c r="I37" s="12">
-        <v>84527.762047507596</v>
+        <v>48085.441416554197</v>
       </c>
       <c r="J37" s="12">
         <v>0</v>
       </c>
       <c r="K37" s="12">
-        <v>1483763.0897349033</v>
+        <v>4437633.2326079691</v>
       </c>
       <c r="L37" s="12">
         <v>0</v>
       </c>
       <c r="M37" s="12">
-        <v>3072.5259449780519</v>
+        <v>9260.197809717527</v>
       </c>
       <c r="N37" s="12">
-        <v>153.46866815595405</v>
+        <v>462.53481668425144</v>
       </c>
       <c r="O37" s="12">
-        <v>28705.64550091168</v>
+        <v>25772.308024303493</v>
       </c>
       <c r="P37" s="12">
-        <v>77989.352880986713</v>
+        <v>342081.03236620937</v>
       </c>
       <c r="Q37" s="12">
-        <v>3888.9872982908187</v>
+        <v>17051.687363539495</v>
       </c>
       <c r="R37" s="12">
-        <v>223183.38656062094</v>
+        <v>216014.55009143314</v>
       </c>
       <c r="S37" s="12">
-        <v>749341.77695455309</v>
+        <v>3837917.1057723179</v>
       </c>
       <c r="T37" s="12">
-        <v>37348.556144635957</v>
+        <v>191213.9251359851</v>
       </c>
       <c r="U37" s="12">
-        <v>1107923.457075953</v>
+        <v>1199055.6164138624</v>
       </c>
       <c r="V37" s="13">
-        <v>0</v>
+        <v>0.8496899585045119</v>
       </c>
       <c r="W37" s="13"/>
       <c r="X37" s="5">
@@ -5411,7 +5412,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A38" s="8">
         <v>43</v>
       </c>
@@ -5422,61 +5423,61 @@
         <v>1.205E-4</v>
       </c>
       <c r="D38" s="11">
-        <v>0.02</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E38" s="10">
         <v>0</v>
       </c>
       <c r="F38" s="12">
-        <v>4137158.869097298</v>
+        <v>7957112.3180603115</v>
       </c>
       <c r="G38" s="12">
-        <v>9870.2526272266605</v>
+        <v>19117.958838042199</v>
       </c>
       <c r="H38" s="12">
-        <v>492.94764873637899</v>
+        <v>954.80361179972999</v>
       </c>
       <c r="I38" s="12">
-        <v>82638.492584021602</v>
+        <v>47682.270956377099</v>
       </c>
       <c r="J38" s="12">
         <v>0</v>
       </c>
       <c r="K38" s="12">
-        <v>1415040.8793178818</v>
+        <v>4339382.1208300134</v>
       </c>
       <c r="L38" s="12">
         <v>0</v>
       </c>
       <c r="M38" s="12">
-        <v>3269.3435444341162</v>
+        <v>10103.162326997513</v>
       </c>
       <c r="N38" s="12">
-        <v>163.28003689537658</v>
+        <v>504.57980175273036</v>
       </c>
       <c r="O38" s="12">
-        <v>27372.513395054899</v>
+        <v>25198.386902766775</v>
       </c>
       <c r="P38" s="12">
-        <v>74916.826936008656</v>
+        <v>332820.83455649187</v>
       </c>
       <c r="Q38" s="12">
-        <v>3735.5186301348645</v>
+        <v>16589.152546855243</v>
       </c>
       <c r="R38" s="12">
-        <v>194477.74105970925</v>
+        <v>190242.24206712961</v>
       </c>
       <c r="S38" s="12">
-        <v>671352.42407356633</v>
+        <v>3495836.0734061087</v>
       </c>
       <c r="T38" s="12">
-        <v>33459.56884634513</v>
+        <v>174162.2377724456</v>
       </c>
       <c r="U38" s="12">
-        <v>884740.07051533216</v>
+        <v>983041.06632242934</v>
       </c>
       <c r="V38" s="13">
-        <v>0</v>
+        <v>0.85676180734698226</v>
       </c>
       <c r="W38" s="13"/>
       <c r="X38" s="5">
@@ -5558,7 +5559,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A39" s="8">
         <v>44</v>
       </c>
@@ -5569,61 +5570,61 @@
         <v>1.35E-4</v>
       </c>
       <c r="D39" s="11">
-        <v>0.02</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E39" s="10">
         <v>0</v>
       </c>
       <c r="F39" s="12">
-        <v>4044157.1762373135</v>
+        <v>7889357.284654092</v>
       </c>
       <c r="G39" s="12">
-        <v>10809.302454913401</v>
+        <v>21235.927352701299</v>
       </c>
       <c r="H39" s="12">
-        <v>539.77192943520095</v>
+        <v>1060.43452186898</v>
       </c>
       <c r="I39" s="12">
-        <v>80768.499039276401</v>
+        <v>47269.049037724697</v>
       </c>
       <c r="J39" s="12">
         <v>0</v>
       </c>
       <c r="K39" s="12">
-        <v>1349146.6461915351</v>
+        <v>4242190.1746704979</v>
       </c>
       <c r="L39" s="12">
         <v>0</v>
       </c>
       <c r="M39" s="12">
-        <v>3492.1613651384359</v>
+        <v>11065.298704463075</v>
       </c>
       <c r="N39" s="12">
-        <v>174.38411829275992</v>
+        <v>552.55532504504106</v>
       </c>
       <c r="O39" s="12">
-        <v>26093.879141754627</v>
+        <v>24630.24752304038</v>
       </c>
       <c r="P39" s="12">
-        <v>71647.483391574526</v>
+        <v>322717.67222949426</v>
       </c>
       <c r="Q39" s="12">
-        <v>3572.2385932394877</v>
+        <v>16084.57274510251</v>
       </c>
       <c r="R39" s="12">
-        <v>167105.22766465435</v>
+        <v>165043.85516436285</v>
       </c>
       <c r="S39" s="12">
-        <v>596435.59713755758</v>
+        <v>3163015.2388496171</v>
       </c>
       <c r="T39" s="12">
-        <v>29724.050216210264</v>
+        <v>157573.08522559036</v>
       </c>
       <c r="U39" s="12">
-        <v>690262.3294556227</v>
+        <v>792798.82425529975</v>
       </c>
       <c r="V39" s="13">
-        <v>0</v>
+        <v>0.86411981165373142</v>
       </c>
       <c r="W39" s="13"/>
       <c r="X39" s="5">
@@ -5705,7 +5706,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="40" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A40" s="8">
         <v>45</v>
       </c>
@@ -5716,61 +5717,61 @@
         <v>1.5100000000000001E-4</v>
       </c>
       <c r="D40" s="11">
-        <v>0.02</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E40" s="10">
         <v>0</v>
       </c>
       <c r="F40" s="12">
-        <v>3952039.6028136881</v>
+        <v>7819791.8737417972</v>
       </c>
       <c r="G40" s="12">
-        <v>11814.915910988</v>
+        <v>23554.953496785201</v>
       </c>
       <c r="H40" s="12">
-        <v>589.89830672027904</v>
+        <v>1176.05806823441</v>
       </c>
       <c r="I40" s="12">
-        <v>78915.481891514006</v>
+        <v>39036.972426106797</v>
       </c>
       <c r="J40" s="12">
         <v>0</v>
       </c>
       <c r="K40" s="12">
-        <v>1285928.3287241119</v>
+        <v>4145909.3897709502</v>
       </c>
       <c r="L40" s="12">
         <v>0</v>
       </c>
       <c r="M40" s="12">
-        <v>3722.9878013990915</v>
+        <v>12101.808177440884</v>
       </c>
       <c r="N40" s="12">
-        <v>185.88233860751419</v>
+        <v>604.22234114140645</v>
       </c>
       <c r="O40" s="12">
-        <v>24866.988359214563</v>
+        <v>20055.991712879819</v>
       </c>
       <c r="P40" s="12">
-        <v>68155.322026436101</v>
+        <v>311652.37352503126</v>
       </c>
       <c r="Q40" s="12">
-        <v>3397.8544749467278</v>
+        <v>15532.017420057471</v>
       </c>
       <c r="R40" s="12">
-        <v>141011.34852289973</v>
+        <v>140413.60764132248</v>
       </c>
       <c r="S40" s="12">
-        <v>524788.11374598288</v>
+        <v>2840297.5666201222</v>
       </c>
       <c r="T40" s="12">
-        <v>26151.811622970774</v>
+        <v>141488.5124804879</v>
       </c>
       <c r="U40" s="12">
-        <v>523157.10179096833</v>
+        <v>627754.96909093671</v>
       </c>
       <c r="V40" s="13">
-        <v>0</v>
+        <v>0.87180708143606411</v>
       </c>
       <c r="W40" s="13"/>
       <c r="X40" s="5">
@@ -5852,7 +5853,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="41" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A41" s="8">
         <v>46</v>
       </c>
@@ -5863,61 +5864,61 @@
         <v>1.6900000000000002E-4</v>
       </c>
       <c r="D41" s="11">
-        <v>0.02</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E41" s="10">
         <v>0</v>
       </c>
       <c r="F41" s="12">
-        <v>3860719.3067044658</v>
+        <v>7756023.8897506706</v>
       </c>
       <c r="G41" s="12">
-        <v>12917.6473106537</v>
+        <v>26147.612685500699</v>
       </c>
       <c r="H41" s="12">
-        <v>644.84531376394796</v>
+        <v>1305.2814572862501</v>
       </c>
       <c r="I41" s="12">
-        <v>77077.380232494805</v>
+        <v>38711.309664786502</v>
       </c>
       <c r="J41" s="12">
         <v>0</v>
       </c>
       <c r="K41" s="12">
-        <v>1225259.411841359</v>
+        <v>4054523.7851398569</v>
       </c>
       <c r="L41" s="12">
         <v>0</v>
       </c>
       <c r="M41" s="12">
-        <v>3970.1667238390046</v>
+        <v>13245.737966737297</v>
       </c>
       <c r="N41" s="12">
-        <v>198.18960412533448</v>
+        <v>661.22350686500522</v>
       </c>
       <c r="O41" s="12">
-        <v>23689.302146170103</v>
+        <v>19610.198083334821</v>
       </c>
       <c r="P41" s="12">
-        <v>64432.334225037004</v>
+        <v>299550.56534759037</v>
       </c>
       <c r="Q41" s="12">
-        <v>3211.9721363392141</v>
+        <v>14927.795078916064</v>
       </c>
       <c r="R41" s="12">
-        <v>116144.36016368517</v>
+        <v>120357.61592844265</v>
       </c>
       <c r="S41" s="12">
-        <v>456632.79171954677</v>
+        <v>2528645.1930950913</v>
       </c>
       <c r="T41" s="12">
-        <v>22753.957148024048</v>
+        <v>125956.4950604304</v>
       </c>
       <c r="U41" s="12">
-        <v>382145.75326806854</v>
+        <v>487341.36144961434</v>
       </c>
       <c r="V41" s="13">
-        <v>0</v>
+        <v>0.87897484945774729</v>
       </c>
       <c r="W41" s="13"/>
       <c r="X41" s="5">
@@ -5999,7 +6000,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A42" s="8">
         <v>47</v>
       </c>
@@ -6010,61 +6011,61 @@
         <v>1.885E-4</v>
       </c>
       <c r="D42" s="11">
-        <v>0.02</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E42" s="10">
         <v>0</v>
       </c>
       <c r="F42" s="12">
-        <v>3770079.4338475531</v>
+        <v>7689859.6859430969</v>
       </c>
       <c r="G42" s="12">
-        <v>14069.7412728401</v>
+        <v>28915.568539247601</v>
       </c>
       <c r="H42" s="12">
-        <v>702.22717543832402</v>
+        <v>1443.1891552054401</v>
       </c>
       <c r="I42" s="12">
-        <v>75252.363478502695</v>
+        <v>38373.204486748902</v>
       </c>
       <c r="J42" s="12">
         <v>0</v>
       </c>
       <c r="K42" s="12">
-        <v>1167010.2335547737</v>
+        <v>3963649.398348562</v>
       </c>
       <c r="L42" s="12">
         <v>0</v>
       </c>
       <c r="M42" s="12">
-        <v>4217.7008903604619</v>
+        <v>14442.81852713588</v>
       </c>
       <c r="N42" s="12">
-        <v>210.50736652840166</v>
+        <v>720.84763059979855</v>
       </c>
       <c r="O42" s="12">
-        <v>22558.478815647875</v>
+        <v>19166.741541136988</v>
       </c>
       <c r="P42" s="12">
-        <v>60462.167501197997</v>
+        <v>286304.82738085306</v>
       </c>
       <c r="Q42" s="12">
-        <v>3013.7825322138797</v>
+        <v>14266.571572051058</v>
       </c>
       <c r="R42" s="12">
-        <v>92455.058017515068</v>
+        <v>100747.41784510783</v>
       </c>
       <c r="S42" s="12">
-        <v>392200.45749450976</v>
+        <v>2229094.6277474998</v>
       </c>
       <c r="T42" s="12">
-        <v>19541.985011684832</v>
+        <v>111028.69998151435</v>
       </c>
       <c r="U42" s="12">
-        <v>266001.39310438349</v>
+        <v>366983.74552117166</v>
       </c>
       <c r="V42" s="13">
-        <v>0</v>
+        <v>0.88653762348177312</v>
       </c>
       <c r="W42" s="13"/>
       <c r="X42" s="5">
@@ -6146,7 +6147,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A43" s="8">
         <v>48</v>
       </c>
@@ -6157,61 +6158,61 @@
         <v>2.0899999999999998E-4</v>
       </c>
       <c r="D43" s="11">
-        <v>0.02</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E43" s="10">
         <v>0</v>
       </c>
       <c r="F43" s="12">
-        <v>3680055.1019207719</v>
+        <v>7621127.7237618947</v>
       </c>
       <c r="G43" s="12">
-        <v>15227.212612748201</v>
+        <v>31773.352438272399</v>
       </c>
       <c r="H43" s="12">
-        <v>759.84879111804798</v>
+        <v>1585.5129926915599</v>
       </c>
       <c r="I43" s="12">
-        <v>73439.600494840794</v>
+        <v>38022.0241173225</v>
       </c>
       <c r="J43" s="12">
         <v>0</v>
       </c>
       <c r="K43" s="12">
-        <v>1111073.6014393794</v>
+        <v>3873219.9438823657</v>
       </c>
       <c r="L43" s="12">
         <v>0</v>
       </c>
       <c r="M43" s="12">
-        <v>4452.197501876899</v>
+        <v>15648.01886930961</v>
       </c>
       <c r="N43" s="12">
-        <v>222.1678369938642</v>
+        <v>780.84732403900125</v>
       </c>
       <c r="O43" s="12">
-        <v>21472.58425932996</v>
+        <v>18725.419421607548</v>
       </c>
       <c r="P43" s="12">
-        <v>56244.466610837539</v>
+        <v>271862.00885371718</v>
       </c>
       <c r="Q43" s="12">
-        <v>2803.275165685478</v>
+        <v>13545.723941451261</v>
       </c>
       <c r="R43" s="12">
-        <v>69896.579201867193</v>
+        <v>81580.676303970846</v>
       </c>
       <c r="S43" s="12">
-        <v>331738.28999331174</v>
+        <v>1942789.8003666468</v>
       </c>
       <c r="T43" s="12">
-        <v>16528.202479470958</v>
+        <v>96762.128409463287</v>
       </c>
       <c r="U43" s="12">
-        <v>173546.33508686844</v>
+        <v>266236.32767606381</v>
       </c>
       <c r="V43" s="13">
-        <v>0</v>
+        <v>0.89453295863661875</v>
       </c>
       <c r="W43" s="13"/>
       <c r="X43" s="5">
@@ -6293,7 +6294,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A44" s="8">
         <v>49</v>
       </c>
@@ -6304,61 +6305,61 @@
         <v>2.3050000000000002E-4</v>
       </c>
       <c r="D44" s="11">
-        <v>0.02</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="E44" s="10">
         <v>0</v>
       </c>
       <c r="F44" s="12">
-        <v>3590628.4400220648</v>
+        <v>7549746.8342136089</v>
       </c>
       <c r="G44" s="12">
-        <v>16385.380504648601</v>
+        <v>34730.721062944598</v>
       </c>
       <c r="H44" s="12">
-        <v>817.47482410274802</v>
+        <v>1732.7330350270099</v>
       </c>
       <c r="I44" s="12">
-        <v>71638.783507900705</v>
+        <v>30125.9062601511</v>
       </c>
       <c r="J44" s="12">
         <v>0</v>
       </c>
       <c r="K44" s="12">
-        <v>1057361.0736673556</v>
+        <v>3783218.3761155871</v>
       </c>
       <c r="L44" s="12">
         <v>0</v>
       </c>
       <c r="M44" s="12">
-        <v>4672.7751640787264</v>
+        <v>16864.995263713583</v>
       </c>
       <c r="N44" s="12">
-        <v>233.12708876325649</v>
+        <v>841.40304418237702</v>
       </c>
       <c r="O44" s="12">
-        <v>20429.91484180429</v>
+        <v>14628.929398606946</v>
       </c>
       <c r="P44" s="12">
-        <v>51792.269108960638</v>
+        <v>256213.98998440756</v>
       </c>
       <c r="Q44" s="12">
-        <v>2581.1073286916135</v>
+        <v>12764.876617412259</v>
       </c>
       <c r="R44" s="12">
-        <v>48423.994942537232</v>
+        <v>62855.256882363297</v>
       </c>
       <c r="S44" s="12">
-        <v>275493.82338247425</v>
+        <v>1670927.7915129298</v>
       </c>
       <c r="T44" s="12">
-        <v>13724.927313785478</v>
+        <v>83216.404468012013</v>
       </c>
       <c r="U44" s="12">
-        <v>103649.75588500126</v>
+        <v>184655.65137209295</v>
       </c>
       <c r="V44" s="13">
-        <v>0</v>
+        <v>0.90299053472756496</v>
       </c>
       <c r="W44" s="13"/>
       <c r="X44" s="5">
@@ -6440,7 +6441,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A45" s="8">
         <v>50</v>
       </c>
@@ -6451,61 +6452,61 @@
         <v>2.5400000000000005E-4</v>
       </c>
       <c r="D45" s="11">
-        <v>0.01</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="E45" s="10">
         <v>0</v>
       </c>
       <c r="F45" s="12">
-        <v>3501786.8011854128</v>
+        <v>7483157.4738554861</v>
       </c>
       <c r="G45" s="12">
-        <v>17697.883648563002</v>
+        <v>37933.5929090434</v>
       </c>
       <c r="H45" s="12">
-        <v>882.75866155480003</v>
+        <v>1892.10237615449</v>
       </c>
       <c r="I45" s="12">
-        <v>34924.486653930398</v>
+        <v>29852.809227158599</v>
       </c>
       <c r="J45" s="12">
         <v>0</v>
       </c>
       <c r="K45" s="12">
-        <v>1005789.0355181949</v>
+        <v>3697345.2746415199</v>
       </c>
       <c r="L45" s="12">
         <v>0</v>
       </c>
       <c r="M45" s="12">
-        <v>4922.7075219190547</v>
+        <v>18162.369432053238</v>
       </c>
       <c r="N45" s="12">
-        <v>245.5413759954204</v>
+        <v>905.92690340152171</v>
       </c>
       <c r="O45" s="12">
-        <v>9714.3272362073785</v>
+        <v>14293.340234560321</v>
       </c>
       <c r="P45" s="12">
-        <v>47119.49394488192</v>
+        <v>239348.994720694</v>
       </c>
       <c r="Q45" s="12">
-        <v>2347.9802399283572</v>
+        <v>11923.47357322988</v>
       </c>
       <c r="R45" s="12">
-        <v>27994.080100732943</v>
+        <v>48226.327483756351</v>
       </c>
       <c r="S45" s="12">
-        <v>223701.55427351364</v>
+        <v>1414713.8015285223</v>
       </c>
       <c r="T45" s="12">
-        <v>11143.819985093864</v>
+        <v>70451.52785059977</v>
       </c>
       <c r="U45" s="12">
-        <v>55225.760942464025</v>
+        <v>121800.39448972965</v>
       </c>
       <c r="V45" s="13">
-        <v>0</v>
+        <v>0.9110258543539429</v>
       </c>
       <c r="W45" s="13"/>
       <c r="X45" s="5">
@@ -6587,7 +6588,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="46" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A46" s="8">
         <v>51</v>
       </c>
@@ -6598,61 +6599,61 @@
         <v>2.7799999999999998E-4</v>
       </c>
       <c r="D46" s="11">
-        <v>0.01</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="E46" s="10">
         <v>0</v>
       </c>
       <c r="F46" s="12">
-        <v>3448281.6722213645</v>
+        <v>7413478.9693431295</v>
       </c>
       <c r="G46" s="12">
-        <v>19073.932221905499</v>
+        <v>41130.787209188202</v>
       </c>
       <c r="H46" s="12">
-        <v>951.17754819563004</v>
+        <v>2051.1072849499401</v>
       </c>
       <c r="I46" s="12">
-        <v>34382.174705051497</v>
+        <v>29567.3675557926</v>
       </c>
       <c r="J46" s="12">
         <v>0</v>
       </c>
       <c r="K46" s="12">
-        <v>966015.89673893445</v>
+        <v>3611630.2898459095</v>
       </c>
       <c r="L46" s="12">
         <v>0</v>
       </c>
       <c r="M46" s="12">
-        <v>5174.7250197180174</v>
+        <v>19417.425615756616</v>
       </c>
       <c r="N46" s="12">
-        <v>258.05283355202403</v>
+        <v>968.30685327984622</v>
       </c>
       <c r="O46" s="12">
-        <v>9327.8248873200482</v>
+        <v>13958.453001358681</v>
       </c>
       <c r="P46" s="12">
-        <v>42196.786422962861</v>
+        <v>221186.62528864076</v>
       </c>
       <c r="Q46" s="12">
-        <v>2102.4388639329368</v>
+        <v>11017.54666982836</v>
       </c>
       <c r="R46" s="12">
-        <v>18279.752864525562</v>
+        <v>33932.987249196027</v>
       </c>
       <c r="S46" s="12">
-        <v>176582.06032863169</v>
+        <v>1175364.8068078284</v>
       </c>
       <c r="T46" s="12">
-        <v>8795.8397451655073</v>
+        <v>58528.054277369898</v>
       </c>
       <c r="U46" s="12">
-        <v>27231.680841731075</v>
+        <v>73574.067005973295</v>
       </c>
       <c r="V46" s="13">
-        <v>0</v>
+        <v>0.91958848997562315</v>
       </c>
       <c r="W46" s="13"/>
       <c r="X46" s="5">
@@ -6734,7 +6735,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A47" s="8">
         <v>52</v>
       </c>
@@ -6745,61 +6746,61 @@
         <v>3.0450000000000003E-4</v>
       </c>
       <c r="D47" s="11">
-        <v>0.01</v>
+        <v>2E-3</v>
       </c>
       <c r="E47" s="10">
         <v>0</v>
       </c>
       <c r="F47" s="12">
-        <v>3393874.3877462121</v>
+        <v>7340729.7072931984</v>
       </c>
       <c r="G47" s="12">
-        <v>20562.220471494598</v>
+        <v>44653.539336904701</v>
       </c>
       <c r="H47" s="12">
-        <v>1025.13650254046</v>
+        <v>2226.2174070814199</v>
       </c>
       <c r="I47" s="12">
-        <v>33830.248962644</v>
+        <v>14634.525924816</v>
       </c>
       <c r="J47" s="12">
         <v>0</v>
       </c>
       <c r="K47" s="12">
-        <v>927345.66826127237</v>
+        <v>3526115.7333900407</v>
       </c>
       <c r="L47" s="12">
         <v>0</v>
       </c>
       <c r="M47" s="12">
-        <v>5441.0334643264296</v>
+        <v>20785.315388529518</v>
       </c>
       <c r="N47" s="12">
-        <v>271.26457590305989</v>
+        <v>1036.2589755876058</v>
       </c>
       <c r="O47" s="12">
-        <v>8951.9279772055143</v>
+        <v>6812.0745057607246</v>
       </c>
       <c r="P47" s="12">
-        <v>37022.06140324485</v>
+        <v>201769.19967288416</v>
       </c>
       <c r="Q47" s="12">
-        <v>1844.3860303809126</v>
+        <v>10049.239816548512</v>
       </c>
       <c r="R47" s="12">
-        <v>8951.9279772055143</v>
+        <v>19974.53424783735</v>
       </c>
       <c r="S47" s="12">
-        <v>134385.27390566884</v>
+        <v>954178.18151918752</v>
       </c>
       <c r="T47" s="12">
-        <v>6693.4008812325701</v>
+        <v>47510.507607541527</v>
       </c>
       <c r="U47" s="12">
-        <v>8951.9279772055143</v>
+        <v>39641.079756777275</v>
       </c>
       <c r="V47" s="13">
-        <v>0</v>
+        <v>0.92870194145836482</v>
       </c>
       <c r="W47" s="13"/>
       <c r="X47" s="5">
@@ -6881,7 +6882,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A48" s="8">
         <v>53</v>
       </c>
@@ -6891,59 +6892,62 @@
       <c r="C48" s="10">
         <v>3.3350000000000003E-4</v>
       </c>
+      <c r="D48">
+        <v>2E-3</v>
+      </c>
       <c r="E48" s="10">
         <v>0</v>
       </c>
       <c r="F48" s="12">
-        <v>3338456.7818095325</v>
+        <v>7279215.4246243965</v>
       </c>
       <c r="G48" s="12">
-        <v>22263.793627921601</v>
+        <v>48495.726504291997</v>
       </c>
       <c r="H48" s="12">
-        <v>1109.66222998547</v>
+        <v>2417.1027146976899</v>
       </c>
       <c r="I48" s="12">
-        <v>0</v>
+        <v>14507.458960129599</v>
       </c>
       <c r="J48" s="12">
         <v>0</v>
       </c>
       <c r="K48" s="12">
-        <v>889725.39293178706</v>
+        <v>3447608.9864783594</v>
       </c>
       <c r="L48" s="12">
         <v>0</v>
       </c>
       <c r="M48" s="12">
-        <v>5746.1227224321447</v>
+        <v>22257.700962840161</v>
       </c>
       <c r="N48" s="12">
-        <v>286.39572664505869</v>
+        <v>1109.3585620466779</v>
       </c>
       <c r="O48" s="12">
-        <v>0</v>
+        <v>6658.3739752133206</v>
       </c>
       <c r="P48" s="12">
-        <v>31581.027938918418</v>
+        <v>180983.88428435463</v>
       </c>
       <c r="Q48" s="12">
-        <v>1573.1214544778527</v>
+        <v>9012.9808409609068</v>
       </c>
       <c r="R48" s="12">
-        <v>0</v>
+        <v>13162.459742076622</v>
       </c>
       <c r="S48" s="12">
-        <v>97363.212502424009</v>
+        <v>752408.98184630345</v>
       </c>
       <c r="T48" s="12">
-        <v>4849.0148508516568</v>
+        <v>37461.267790993021</v>
       </c>
       <c r="U48" s="12">
-        <v>0</v>
+        <v>19666.545508939926</v>
       </c>
       <c r="V48" s="13">
-        <v>0</v>
+        <v>0.93655009959209434</v>
       </c>
       <c r="W48" s="13"/>
       <c r="X48" s="5">
@@ -7025,7 +7029,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="49" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A49" s="8">
         <v>54</v>
       </c>
@@ -7035,59 +7039,62 @@
       <c r="C49" s="10">
         <v>3.6350000000000005E-4</v>
       </c>
+      <c r="D49">
+        <v>2E-3</v>
+      </c>
       <c r="E49" s="10">
         <v>0</v>
       </c>
       <c r="F49" s="12">
-        <v>3315083.3259516256</v>
+        <v>7213795.1364452764</v>
       </c>
       <c r="G49" s="12">
-        <v>24096.275485480401</v>
+        <v>52382.324133240902</v>
       </c>
       <c r="H49" s="12">
-        <v>1200.6524947954599</v>
+        <v>2610.07009949141</v>
       </c>
       <c r="I49" s="12">
-        <v>0</v>
+        <v>14372.5332994663</v>
       </c>
       <c r="J49" s="12">
         <v>0</v>
       </c>
       <c r="K49" s="12">
-        <v>861725.64968318772</v>
+        <v>3368785.3435712978</v>
       </c>
       <c r="L49" s="12">
         <v>0</v>
       </c>
       <c r="M49" s="12">
-        <v>6065.8266257814457</v>
+        <v>23704.876637362428</v>
       </c>
       <c r="N49" s="12">
-        <v>302.24380011050584</v>
+        <v>1181.1501445780573</v>
       </c>
       <c r="O49" s="12">
-        <v>0</v>
+        <v>6504.0857668633025</v>
       </c>
       <c r="P49" s="12">
-        <v>25834.90521648627</v>
+        <v>158726.18332151446</v>
       </c>
       <c r="Q49" s="12">
-        <v>1286.7257278327941</v>
+        <v>7903.6222789142284</v>
       </c>
       <c r="R49" s="12">
-        <v>0</v>
+        <v>6504.0857668633025</v>
       </c>
       <c r="S49" s="12">
-        <v>65782.18456350558</v>
+        <v>571425.09756194882</v>
       </c>
       <c r="T49" s="12">
-        <v>3275.893396373805</v>
+        <v>28448.286950032118</v>
       </c>
       <c r="U49" s="12">
-        <v>0</v>
+        <v>6504.0857668633025</v>
       </c>
       <c r="V49" s="13">
-        <v>0</v>
+        <v>0.94504346213575119</v>
       </c>
       <c r="W49" s="13"/>
       <c r="X49" s="5">
@@ -7169,7 +7176,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="50" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A50" s="8">
         <v>55</v>
       </c>
@@ -7183,13 +7190,13 @@
         <v>0</v>
       </c>
       <c r="F50" s="12">
-        <v>3289786.3979713498</v>
+        <v>7144430.2089130776</v>
       </c>
       <c r="G50" s="12">
-        <v>25951.294777198302</v>
+        <v>56358.435453728998</v>
       </c>
       <c r="H50" s="12">
-        <v>1292.70083120407</v>
+        <v>2807.3588228210001</v>
       </c>
       <c r="I50" s="12">
         <v>0</v>
@@ -7198,40 +7205,40 @@
         <v>0</v>
       </c>
       <c r="K50" s="12">
-        <v>834077.90283563093</v>
+        <v>3289676.8216174771</v>
       </c>
       <c r="L50" s="12">
         <v>0</v>
       </c>
       <c r="M50" s="12">
-        <v>6371.8192567882807</v>
+        <v>25147.103355842686</v>
       </c>
       <c r="N50" s="12">
-        <v>317.39672799561021</v>
+        <v>1252.6419852867907</v>
       </c>
       <c r="O50" s="12">
         <v>0</v>
       </c>
       <c r="P50" s="12">
-        <v>19769.078590704827</v>
+        <v>135021.30668415205</v>
       </c>
       <c r="Q50" s="12">
-        <v>984.48192772228822</v>
+        <v>6722.4721343361707</v>
       </c>
       <c r="R50" s="12">
         <v>0</v>
       </c>
       <c r="S50" s="12">
-        <v>39947.279347019314</v>
+        <v>412698.91424043442</v>
       </c>
       <c r="T50" s="12">
-        <v>1989.1676685410107</v>
+        <v>20544.664671117887</v>
       </c>
       <c r="U50" s="12">
         <v>0</v>
       </c>
       <c r="V50" s="13">
-        <v>0</v>
+        <v>0.95421884342564656</v>
       </c>
       <c r="W50" s="13"/>
       <c r="X50" s="5">
@@ -7313,7 +7320,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A51" s="8">
         <v>56</v>
       </c>
@@ -7327,13 +7334,13 @@
         <v>0</v>
       </c>
       <c r="F51" s="12">
-        <v>3262542.4023629474</v>
+        <v>7085264.4146365281</v>
       </c>
       <c r="G51" s="12">
-        <v>27627.8827048083</v>
+        <v>59999.482010825297</v>
       </c>
       <c r="H51" s="12">
-        <v>1375.83526419487</v>
+        <v>2987.90189845247</v>
       </c>
       <c r="I51" s="12">
         <v>0</v>
@@ -7342,40 +7349,40 @@
         <v>0</v>
       </c>
       <c r="K51" s="12">
-        <v>806787.98830610455</v>
+        <v>3216753.6434485549</v>
       </c>
       <c r="L51" s="12">
         <v>0</v>
       </c>
       <c r="M51" s="12">
-        <v>6616.3179115186085</v>
+        <v>26396.882665431545</v>
       </c>
       <c r="N51" s="12">
-        <v>329.48465863463338</v>
+        <v>1314.5329457184282</v>
       </c>
       <c r="O51" s="12">
         <v>0</v>
       </c>
       <c r="P51" s="12">
-        <v>13397.259333916545</v>
+        <v>109874.20332830936</v>
       </c>
       <c r="Q51" s="12">
-        <v>667.08519972667796</v>
+        <v>5469.8301490493805</v>
       </c>
       <c r="R51" s="12">
         <v>0</v>
       </c>
       <c r="S51" s="12">
-        <v>20178.20075631448</v>
+        <v>277677.60755628237</v>
       </c>
       <c r="T51" s="12">
-        <v>1004.6857408187225</v>
+        <v>13822.192536781715</v>
       </c>
       <c r="U51" s="12">
         <v>0</v>
       </c>
       <c r="V51" s="13">
-        <v>0</v>
+        <v>0.96218708744323067</v>
       </c>
       <c r="W51" s="14"/>
       <c r="X51" s="5">
@@ -7457,7 +7464,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="52" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A52" s="8">
         <v>57</v>
       </c>
@@ -7471,13 +7478,13 @@
         <v>0</v>
       </c>
       <c r="F52" s="12">
-        <v>3233538.6843939442</v>
+        <v>7022277.0307272505</v>
       </c>
       <c r="G52" s="12">
-        <v>29030.658539534499</v>
+        <v>63045.890755214001</v>
       </c>
       <c r="H52" s="12">
-        <v>1445.34002296976</v>
+        <v>3138.8454060798199</v>
       </c>
       <c r="I52" s="12">
         <v>0</v>
@@ -7486,40 +7493,40 @@
         <v>0</v>
       </c>
       <c r="K52" s="12">
-        <v>779912.10989799199</v>
+        <v>3143516.9050618652</v>
       </c>
       <c r="L52" s="12">
         <v>0</v>
       </c>
       <c r="M52" s="12">
-        <v>6780.9414223979365</v>
+        <v>27348.784461850504</v>
       </c>
       <c r="N52" s="12">
-        <v>337.60054109204458</v>
+        <v>1361.6051013260876</v>
       </c>
       <c r="O52" s="12">
         <v>0</v>
       </c>
       <c r="P52" s="12">
-        <v>6780.9414223979365</v>
+        <v>83477.320662877813</v>
       </c>
       <c r="Q52" s="12">
-        <v>337.60054109204458</v>
+        <v>4155.2972033309525</v>
       </c>
       <c r="R52" s="12">
         <v>0</v>
       </c>
       <c r="S52" s="12">
-        <v>6780.9414223979365</v>
+        <v>167803.40422797299</v>
       </c>
       <c r="T52" s="12">
-        <v>337.60054109204458</v>
+        <v>8352.3623877323353</v>
       </c>
       <c r="U52" s="12">
         <v>0</v>
       </c>
       <c r="V52" s="13">
-        <v>0</v>
+        <v>0.97081757114590228</v>
       </c>
       <c r="W52" s="14"/>
       <c r="X52" s="5">
@@ -7601,68 +7608,70 @@
         <v>43</v>
       </c>
     </row>
-    <row r="53" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A53" s="8">
         <v>58</v>
       </c>
-      <c r="B53" s="15"/>
+      <c r="B53" s="15">
+        <v>9.3900000000000008E-3</v>
+      </c>
       <c r="C53" s="10">
-        <v>0</v>
+        <v>4.6950000000000008E-4</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F53" s="12">
-        <v>3203062.6858314397</v>
+        <v>6956092.294565957</v>
       </c>
       <c r="G53" s="12">
-        <v>0</v>
+        <v>65302.373314339202</v>
       </c>
       <c r="H53" s="12">
-        <v>0</v>
+        <v>3250.5520006635702</v>
       </c>
       <c r="I53" s="12">
         <v>0</v>
       </c>
       <c r="J53" s="12">
-        <v>3203062.6858314401</v>
+        <v>0</v>
       </c>
       <c r="K53" s="12">
-        <v>753524.51281640865</v>
+        <v>3070289.1641244171</v>
       </c>
       <c r="L53" s="12">
-        <v>753524.51281640877</v>
+        <v>0</v>
       </c>
       <c r="M53" s="12">
-        <v>0</v>
+        <v>27930.98883695943</v>
       </c>
       <c r="N53" s="12">
-        <v>0</v>
+        <v>1390.3190196083465</v>
       </c>
       <c r="O53" s="12">
         <v>0</v>
       </c>
       <c r="P53" s="12">
-        <v>0</v>
+        <v>56128.536201027309</v>
       </c>
       <c r="Q53" s="12">
-        <v>0</v>
+        <v>2793.6921020048649</v>
       </c>
       <c r="R53" s="12">
         <v>0</v>
       </c>
       <c r="S53" s="12">
-        <v>0</v>
+        <v>84326.083565095192</v>
       </c>
       <c r="T53" s="12">
-        <v>0</v>
+        <v>4197.0651844013828</v>
       </c>
       <c r="U53" s="12">
         <v>0</v>
       </c>
       <c r="V53" s="13">
-        <v>0</v>
+        <v>0.98005455393539653</v>
       </c>
       <c r="W53" s="14"/>
       <c r="X53" s="5">
@@ -7744,26 +7753,28 @@
         <v>44</v>
       </c>
     </row>
-    <row r="54" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A54" s="8">
         <v>59</v>
       </c>
-      <c r="B54" s="15"/>
+      <c r="B54" s="15">
+        <v>9.7099999999999999E-3</v>
+      </c>
       <c r="C54" s="10">
-        <v>0</v>
+        <v>4.8550000000000004E-4</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="10">
         <v>0</v>
       </c>
       <c r="F54" s="12">
-        <v>0</v>
+        <v>6887539.3692509541</v>
       </c>
       <c r="G54" s="12">
-        <v>0</v>
+        <v>66861.772639160699</v>
       </c>
       <c r="H54" s="12">
-        <v>0</v>
+        <v>3327.6657275052298</v>
       </c>
       <c r="I54" s="12">
         <v>0</v>
@@ -7772,40 +7783,40 @@
         <v>0</v>
       </c>
       <c r="K54" s="12">
-        <v>0</v>
+        <v>2997465.1397268395</v>
       </c>
       <c r="L54" s="12">
         <v>0</v>
       </c>
       <c r="M54" s="12">
-        <v>0</v>
+        <v>28197.547364067879</v>
       </c>
       <c r="N54" s="12">
-        <v>0</v>
+        <v>1403.3730823965182</v>
       </c>
       <c r="O54" s="12">
         <v>0</v>
       </c>
       <c r="P54" s="12">
-        <v>0</v>
+        <v>28197.547364067879</v>
       </c>
       <c r="Q54" s="12">
-        <v>0</v>
+        <v>1403.3730823965182</v>
       </c>
       <c r="R54" s="12">
         <v>0</v>
       </c>
       <c r="S54" s="12">
-        <v>0</v>
+        <v>28197.547364067879</v>
       </c>
       <c r="T54" s="12">
-        <v>0</v>
+        <v>1403.3730823965182</v>
       </c>
       <c r="U54" s="12">
         <v>0</v>
       </c>
       <c r="V54" s="13">
-        <v>0</v>
+        <v>0.9898092142049999</v>
       </c>
       <c r="W54" s="14"/>
       <c r="X54" s="5">
@@ -7887,7 +7898,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A55" s="8">
         <v>60</v>
       </c>
@@ -7899,10 +7910,10 @@
       </c>
       <c r="D55" s="12"/>
       <c r="E55" s="10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F55" s="12">
-        <v>0</v>
+        <v>6817349.9308842877</v>
       </c>
       <c r="G55" s="12">
         <v>0</v>
@@ -7914,13 +7925,13 @@
         <v>0</v>
       </c>
       <c r="J55" s="12">
-        <v>0</v>
+        <v>6817349.9308842896</v>
       </c>
       <c r="K55" s="12">
-        <v>0</v>
+        <v>2925376.2813133607</v>
       </c>
       <c r="L55" s="12">
-        <v>0</v>
+        <v>2925376.2813133616</v>
       </c>
       <c r="M55" s="12">
         <v>0</v>
@@ -7950,7 +7961,7 @@
         <v>0</v>
       </c>
       <c r="V55" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W55" s="14"/>
       <c r="X55" s="5">
@@ -8032,7 +8043,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="56" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A56" s="8">
         <v>61</v>
       </c>
@@ -8177,7 +8188,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="57" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A57" s="8">
         <v>62</v>
       </c>
@@ -8322,7 +8333,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="58" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A58" s="8">
         <v>63</v>
       </c>
@@ -8467,7 +8478,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="59" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A59" s="8">
         <v>64</v>
       </c>
@@ -8612,7 +8623,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A60" s="8">
         <v>65</v>
       </c>
@@ -8757,7 +8768,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="61" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:50" x14ac:dyDescent="0.3">
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
@@ -8842,7 +8853,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="62" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:50" x14ac:dyDescent="0.3">
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
@@ -8927,7 +8938,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="63" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:50" x14ac:dyDescent="0.3">
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
@@ -9012,7 +9023,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="64" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:50" x14ac:dyDescent="0.3">
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
@@ -9097,7 +9108,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="65" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
@@ -9182,7 +9193,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="66" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
@@ -9267,7 +9278,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="67" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="67" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>
       <c r="E67" s="1"/>
@@ -9352,7 +9363,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="68" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="68" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
       <c r="E68" s="1"/>
@@ -9437,7 +9448,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="69" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
@@ -9522,7 +9533,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="70" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="70" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
       <c r="E70" s="1"/>
@@ -9607,7 +9618,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="71" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="71" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C71" s="1"/>
       <c r="D71" s="1"/>
       <c r="E71" s="1"/>
@@ -9692,7 +9703,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="72" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="72" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
       <c r="E72" s="1"/>
@@ -9777,7 +9788,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="73" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="73" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C73" s="1"/>
       <c r="D73" s="1"/>
       <c r="E73" s="1"/>
@@ -9862,7 +9873,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="74" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
@@ -9947,7 +9958,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="75" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="75" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C75" s="1"/>
       <c r="D75" s="1"/>
       <c r="E75" s="1"/>
@@ -10032,7 +10043,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="76" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="76" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
       <c r="E76" s="1"/>
@@ -10117,7 +10128,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="77" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="77" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
       <c r="E77" s="1"/>
@@ -10202,7 +10213,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="78" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
       <c r="E78" s="1"/>
@@ -10287,7 +10298,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="79" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C79" s="1"/>
       <c r="D79" s="1"/>
       <c r="E79" s="1"/>
@@ -10372,7 +10383,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="80" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="80" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
@@ -10457,7 +10468,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="81" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
       <c r="E81" s="1"/>
@@ -10542,7 +10553,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="82" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="82" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C82" s="1"/>
       <c r="X82" s="5">
         <v>73</v>
@@ -10623,7 +10634,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="83" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C83" s="1"/>
       <c r="X83" s="5">
         <v>74</v>
@@ -10704,7 +10715,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="84" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="84" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C84" s="1"/>
       <c r="X84" s="5">
         <v>75</v>
@@ -10785,7 +10796,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="85" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="85" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C85" s="1"/>
       <c r="X85" s="5">
         <v>76</v>
@@ -10866,7 +10877,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="86" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="86" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C86" s="1"/>
       <c r="X86" s="5">
         <v>77</v>
@@ -10947,7 +10958,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="87" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="87" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C87" s="1"/>
       <c r="X87" s="5">
         <v>78</v>
@@ -11028,7 +11039,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="88" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="88" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C88" s="1"/>
       <c r="X88" s="5">
         <v>79</v>
@@ -11109,7 +11120,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="89" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="89" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C89" s="1"/>
       <c r="X89" s="5">
         <v>80</v>
@@ -11190,7 +11201,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="90" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="90" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C90" s="1"/>
       <c r="X90" s="5">
         <v>81</v>
@@ -11271,7 +11282,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="91" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="91" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C91" s="1"/>
       <c r="X91" s="5">
         <v>82</v>
@@ -11352,7 +11363,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="92" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="92" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C92" s="1"/>
       <c r="X92" s="5">
         <v>83</v>
@@ -11433,7 +11444,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="93" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="93" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C93" s="1"/>
       <c r="X93" s="5">
         <v>84</v>
@@ -11514,7 +11525,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="94" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="94" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C94" s="1"/>
       <c r="X94" s="5">
         <v>85</v>
@@ -11595,7 +11606,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="95" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="95" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C95" s="1"/>
       <c r="X95" s="5">
         <v>86</v>
@@ -11676,7 +11687,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="96" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="96" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C96" s="1"/>
       <c r="X96" s="5">
         <v>87</v>
@@ -11757,7 +11768,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="97" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="97" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C97" s="1"/>
       <c r="X97" s="5">
         <v>88</v>
@@ -11838,7 +11849,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="98" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="98" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C98" s="1"/>
       <c r="X98" s="5">
         <v>89</v>
@@ -11919,7 +11930,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="99" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="99" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C99" s="1"/>
       <c r="X99" s="5">
         <v>90</v>
@@ -12000,7 +12011,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="100" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="100" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C100" s="1"/>
       <c r="X100" s="5">
         <v>91</v>
@@ -12081,7 +12092,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="101" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="101" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C101" s="1"/>
       <c r="X101" s="5">
         <v>92</v>
@@ -12162,7 +12173,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="102" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="102" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C102" s="1"/>
       <c r="X102" s="5">
         <v>93</v>
@@ -12243,7 +12254,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="103" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="103" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C103" s="1"/>
       <c r="X103" s="5">
         <v>94</v>
@@ -12324,7 +12335,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="104" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="104" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C104" s="1"/>
       <c r="X104" s="5">
         <v>95</v>
@@ -12405,7 +12416,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="105" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="105" spans="3:50" x14ac:dyDescent="0.3">
       <c r="C105" s="1"/>
       <c r="X105" s="5">
         <v>96</v>
@@ -12486,7 +12497,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="106" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="106" spans="3:50" x14ac:dyDescent="0.3">
       <c r="X106" s="5">
         <v>97</v>
       </c>
@@ -12566,7 +12577,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="107" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="107" spans="3:50" x14ac:dyDescent="0.3">
       <c r="X107" s="5">
         <v>98</v>
       </c>
@@ -12646,7 +12657,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="108" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="108" spans="3:50" x14ac:dyDescent="0.3">
       <c r="X108" s="5">
         <v>99</v>
       </c>
@@ -12726,7 +12737,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="109" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="109" spans="3:50" x14ac:dyDescent="0.3">
       <c r="X109" s="5">
         <v>100</v>
       </c>
@@ -12806,7 +12817,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="110" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="110" spans="3:50" x14ac:dyDescent="0.3">
       <c r="X110" s="5">
         <v>101</v>
       </c>
@@ -12886,7 +12897,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="111" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="111" spans="3:50" x14ac:dyDescent="0.3">
       <c r="X111" s="5">
         <v>102</v>
       </c>
@@ -12962,7 +12973,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="112" spans="3:50" x14ac:dyDescent="0.25">
+    <row r="112" spans="3:50" x14ac:dyDescent="0.3">
       <c r="X112" s="5">
         <v>103</v>
       </c>
@@ -13038,7 +13049,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="113" spans="24:50" x14ac:dyDescent="0.25">
+    <row r="113" spans="24:50" x14ac:dyDescent="0.3">
       <c r="X113" s="5">
         <v>104</v>
       </c>
@@ -13114,7 +13125,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="114" spans="24:50" x14ac:dyDescent="0.25">
+    <row r="114" spans="24:50" x14ac:dyDescent="0.3">
       <c r="X114" s="5">
         <v>105</v>
       </c>
@@ -13188,7 +13199,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="115" spans="24:50" x14ac:dyDescent="0.25">
+    <row r="115" spans="24:50" x14ac:dyDescent="0.3">
       <c r="X115" s="5">
         <v>106</v>
       </c>
@@ -13262,7 +13273,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="116" spans="24:50" x14ac:dyDescent="0.25">
+    <row r="116" spans="24:50" x14ac:dyDescent="0.3">
       <c r="X116" s="5">
         <v>107</v>
       </c>
@@ -13336,7 +13347,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="117" spans="24:50" x14ac:dyDescent="0.25">
+    <row r="117" spans="24:50" x14ac:dyDescent="0.3">
       <c r="X117" s="5">
         <v>108</v>
       </c>
@@ -13410,7 +13421,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="118" spans="24:50" x14ac:dyDescent="0.25">
+    <row r="118" spans="24:50" x14ac:dyDescent="0.3">
       <c r="X118" s="5">
         <v>109</v>
       </c>
@@ -13484,7 +13495,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="119" spans="24:50" x14ac:dyDescent="0.25">
+    <row r="119" spans="24:50" x14ac:dyDescent="0.3">
       <c r="X119" s="5">
         <v>110</v>
       </c>
@@ -13558,7 +13569,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="120" spans="24:50" x14ac:dyDescent="0.25">
+    <row r="120" spans="24:50" x14ac:dyDescent="0.3">
       <c r="AU120" s="6">
         <v>1</v>
       </c>

</xml_diff>